<commit_message>
produktjakt 2026-09-09: 9 produkter av 22 granskade
Tva sokomgangar (6 + 14 sokord, manad 9). 22 kandidater klarade ekonomin,
13 strokos i lasningen med orsak i korningens STATUS.md: sex dubbletter i
sak, fem regnvattenavledare i fel sasong, en kedjevara utan ankare och en
batreservdel utan payoff.

Sokordet "downpipe rain diverter water butt" flyttat fran manad 9-3 till
en ny grupp pa manad 4-6 — regntunnan kopplas in pa varen, inte nu.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016jBJVGuyny8S3j2XPSM26Z
</commit_message>
<xml_diff>
--- a/produktjakt/korningar/2026-09-09/Leverantorsoffert-2026-09-09.xlsx
+++ b/produktjakt/korningar/2026-09-09/Leverantorsoffert-2026-09-09.xlsx
@@ -732,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU44"/>
+  <dimension ref="A1:AU40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="18" customWidth="1" style="71" min="1" max="1"/>
@@ -767,7 +767,7 @@
   <sheetData>
     <row r="1" ht="27.75" customHeight="1" s="71">
       <c r="A1" s="1" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AP1" s="1" t="n"/>
       <c r="AQ1" s="1" t="n"/>
@@ -1027,17 +1027,17 @@
     </row>
     <row r="5" ht="24" customHeight="1" s="71">
       <c r="A5" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sf82b0d4f34464eaca317489c4e31f25f8.jpg")</f>
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sd362c7c33848404bb3e573470af41733h.jpg")</f>
         <v/>
       </c>
       <c r="D5" s="18" t="inlineStr">
         <is>
-          <t>Professional Telescopic Boat Cover Support Pole Windproof Adjustable H…</t>
+          <t>Flexible Chimney Sweep Set Flue Sweeping Brush &amp; Rod Kit Soot Cleaning…</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $10.77. Vår räkning: landad ca 155 kr, tänkt butikspris 399 kr. Originaltitel: Professional Telescopic Boat Cover Support Pole Windproof Adjustable Height 22"-70" Heavy-Duty Steel/Aluminum for Pontoon Patio</t>
+          <t>AliExpress: US $15.81. Vår räkning: landad ca 228 kr, tänkt butikspris 599 kr. Originaltitel: Flexible Chimney Sweep Set Flue Sweeping Brush &amp; Rod Kit Soot Cleaning Rods Nylon Brush Cleaning Tool Kit</t>
         </is>
       </c>
       <c r="H5" s="13" t="n"/>
@@ -1052,7 +1052,7 @@
       <c r="M5" s="14" t="n"/>
       <c r="N5" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005009100129778.html</t>
+          <t>https://www.aliexpress.com/item/1005008077527346.html</t>
         </is>
       </c>
       <c r="Q5" s="18" t="n"/>
@@ -1200,17 +1200,17 @@
     </row>
     <row r="9" ht="24" customHeight="1" s="71">
       <c r="A9" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S4244c19ccbb7400787c5f68f47dda6f9q.jpg")</f>
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sddf296c4c78d43d7a1d84ca5614acb6fL.jpg")</f>
         <v/>
       </c>
       <c r="D9" s="18" t="inlineStr">
         <is>
-          <t>Solar Powered Marine Signal Lights LED Navigation Warning Lamps Waterp…</t>
+          <t>Foldable Cane Easy To Carry Seat Portable Stool Folding Chair Non Slip…</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $11.00. Vår räkning: landad ca 158 kr, tänkt butikspris 399 kr. Originaltitel: Solar Powered Marine Signal Lights LED Navigation Warning Lamps Waterproof Boat Marker Beacons For Yacht Fishing Vessel</t>
+          <t>AliExpress: US $16.08. Vår räkning: landad ca 232 kr, tänkt butikspris 599 kr. Originaltitel: Foldable Cane Easy To Carry Seat Portable Stool Folding Chair Non Slip Handle Super Light Walking Stick For Outdoor Walking</t>
         </is>
       </c>
       <c r="H9" s="13" t="n"/>
@@ -1225,7 +1225,7 @@
       <c r="M9" s="14" t="n"/>
       <c r="N9" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005011767102250.html</t>
+          <t>https://www.aliexpress.com/item/1005011927514185.html</t>
         </is>
       </c>
       <c r="Q9" s="18" t="n"/>
@@ -1373,17 +1373,17 @@
     </row>
     <row r="13" ht="24" customHeight="1" s="71">
       <c r="A13" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sd45dbbc9fcb64ef4a78670e4fe959d40T.png")</f>
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S20416daaf99f4237ab753083a39afac5H.jpg")</f>
         <v/>
       </c>
       <c r="D13" s="18" t="inlineStr">
         <is>
-          <t>Windshield Sunshade Front Motorhome Thermal Windscreen Screen Cover Fo…</t>
+          <t>Winter Warm Waterproof Stray Cat Dog House Foldable Washable Pet Cave …</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $19.67. Vår räkning: landad ca 283 kr, tänkt butikspris 699 kr. Originaltitel: Windshield Sunshade Front Motorhome Thermal Windscreen Screen Cover For Fiat Ducato Peugeot Boxer Citroen Relay RV Cover</t>
+          <t>AliExpress: US $21.66. Vår räkning: landad ca 312 kr, tänkt butikspris 799 kr. Originaltitel: Winter Warm Waterproof Stray Cat Dog House Foldable Washable Pet Cave Outdoor Shelter Sleeping Bed for Small Puppy Pet Supplies</t>
         </is>
       </c>
       <c r="H13" s="13" t="n"/>
@@ -1398,7 +1398,7 @@
       <c r="M13" s="14" t="n"/>
       <c r="N13" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005011618553986.html</t>
+          <t>https://www.aliexpress.com/item/1005012414077421.html</t>
         </is>
       </c>
       <c r="Q13" s="18" t="n"/>
@@ -1546,17 +1546,17 @@
     </row>
     <row r="17" ht="24" customHeight="1" s="71">
       <c r="A17" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S4d8623aa49aa4b18bfe95b3f674c7ba8T.jpg")</f>
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sf82b0d4f34464eaca317489c4e31f25f8.jpg")</f>
         <v/>
       </c>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>JVEE 30W 1000mAh Solar Flood Lights Remote Control Powered Spotlight O…</t>
+          <t>Professional Telescopic Boat Cover Support Pole Windproof Adjustable H…</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $11.33. Vår räkning: landad ca 163 kr, tänkt butikspris 399 kr. Originaltitel: JVEE 30W 1000mAh Solar Flood Lights Remote Control Powered Spotlight Outdoor Waterproof IP67 Villa Street Lamp Adjustable Angle</t>
+          <t>AliExpress: US $10.77. Vår räkning: landad ca 155 kr, tänkt butikspris 399 kr. Originaltitel: Professional Telescopic Boat Cover Support Pole Windproof Adjustable Height 22"-70" Heavy-Duty Steel/Aluminum for Pontoon Patio</t>
         </is>
       </c>
       <c r="H17" s="13" t="n"/>
@@ -1571,7 +1571,7 @@
       <c r="M17" s="14" t="n"/>
       <c r="N17" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005007487622885.html</t>
+          <t>https://www.aliexpress.com/item/1005009100129778.html</t>
         </is>
       </c>
       <c r="Q17" s="18" t="n"/>
@@ -1719,17 +1719,17 @@
     </row>
     <row r="21" ht="24" customHeight="1" s="71">
       <c r="A21" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S15d605ad9579448ba3c140e67d273f235.jpg")</f>
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S1765e6b203364ba5b2b27145c16238989.jpg")</f>
         <v/>
       </c>
       <c r="D21" s="18" t="inlineStr">
         <is>
-          <t>1/2/3Pcs Solar Charging LED Longshot Warning Light 3 Color Flashing To…</t>
+          <t>Outboard Motor Flusher Muffs Kit with 16mm Quick Connect Fitting, Adju…</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $22.62. Vår räkning: landad ca 326 kr, tänkt butikspris 799 kr. Originaltitel: 1/2/3Pcs Solar Charging LED Longshot Warning Light 3 Color Flashing Torch Light Portable Flashlight Boat Navigation Signal Light</t>
+          <t>AliExpress: US $25.05. Vår räkning: landad ca 361 kr, tänkt butikspris 899 kr. Originaltitel: Outboard Motor Flusher Muffs Kit with 16mm Quick Connect Fitting, Adjustable Dual/Single Tube for Boat Motor Cleaning &amp; Test Run</t>
         </is>
       </c>
       <c r="H21" s="13" t="n"/>
@@ -1744,7 +1744,7 @@
       <c r="M21" s="14" t="n"/>
       <c r="N21" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005010712839288.html</t>
+          <t>https://www.aliexpress.com/item/1005011764722846.html</t>
         </is>
       </c>
       <c r="Q21" s="18" t="n"/>
@@ -1892,17 +1892,17 @@
     </row>
     <row r="25" ht="24" customHeight="1" s="71">
       <c r="A25" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Seabb27633c8549378b013f0e7843e929k.jpg")</f>
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S4f5c23377f414f0c868c1af6496a8f73E.jpg")</f>
         <v/>
       </c>
       <c r="D25" s="18" t="inlineStr">
         <is>
-          <t>FLYY-Water Butt Filler Set For Downpipes, Rainwater Collector, Rain Ba…</t>
+          <t>Roof Ladder Stabilizer, Ladder Standoff, Extension Ladder Stabilizer, …</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $22.64. Vår räkning: landad ca 326 kr, tänkt butikspris 799 kr. Originaltitel: FLYY-Water Butt Filler Set For Downpipes, Rainwater Collector, Rain Barrel Diverter Kit Connects Downpipe To Water Butt</t>
+          <t>AliExpress: US $27.55. Vår räkning: landad ca 397 kr, tänkt butikspris 999 kr. Originaltitel: Roof Ladder Stabilizer, Ladder Standoff, Extension Ladder Stabilizer, Wall Bracket, Heavy Duty Secure</t>
         </is>
       </c>
       <c r="H25" s="13" t="n"/>
@@ -1917,7 +1917,7 @@
       <c r="M25" s="14" t="n"/>
       <c r="N25" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005012797654262.html</t>
+          <t>https://www.aliexpress.com/item/1005012386302696.html</t>
         </is>
       </c>
       <c r="Q25" s="18" t="n"/>
@@ -2065,17 +2065,17 @@
     </row>
     <row r="29" ht="24" customHeight="1" s="71">
       <c r="A29" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S7eb1605108374fc9bbb9c200eb2dc734f.jpg")</f>
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S4244c19ccbb7400787c5f68f47dda6f9q.jpg")</f>
         <v/>
       </c>
       <c r="D29" s="18" t="inlineStr">
         <is>
-          <t>Rainwater Collection System Easy Installation Efficient Rain Barrel Di…</t>
+          <t>Solar Powered Marine Signal Lights LED Navigation Warning Lamps Waterp…</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $20.03. Vår räkning: landad ca 288 kr, tänkt butikspris 699 kr. Originaltitel: Rainwater Collection System Easy Installation Efficient Rain Barrel Diverter Kit For Downspout Brown</t>
+          <t>AliExpress: US $11.00. Vår räkning: landad ca 158 kr, tänkt butikspris 399 kr. Originaltitel: Solar Powered Marine Signal Lights LED Navigation Warning Lamps Waterproof Boat Marker Beacons For Yacht Fishing Vessel</t>
         </is>
       </c>
       <c r="H29" s="13" t="n"/>
@@ -2090,7 +2090,7 @@
       <c r="M29" s="14" t="n"/>
       <c r="N29" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005010580025501.html</t>
+          <t>https://www.aliexpress.com/item/1005011767102250.html</t>
         </is>
       </c>
       <c r="Q29" s="18" t="n"/>
@@ -2238,17 +2238,17 @@
     </row>
     <row r="33" ht="24" customHeight="1" s="71">
       <c r="A33" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S31821eb7745f4de694136cf4e2a6df7cX.jpg")</f>
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sd45dbbc9fcb64ef4a78670e4fe959d40T.png")</f>
         <v/>
       </c>
       <c r="D33" s="18" t="inlineStr">
         <is>
-          <t>3 in 1 Aluminum Ship Boat Cover Support Pole Marine Adjustable Stand 2…</t>
+          <t>Windshield Sunshade Front Motorhome Thermal Windscreen Screen Cover Fo…</t>
         </is>
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $28.81. Vår räkning: landad ca 415 kr, tänkt butikspris 999 kr. Originaltitel: 3 in 1 Aluminum Ship Boat Cover Support Pole Marine Adjustable Stand 22'' to</t>
+          <t>AliExpress: US $19.67. Vår räkning: landad ca 283 kr, tänkt butikspris 699 kr. Originaltitel: Windshield Sunshade Front Motorhome Thermal Windscreen Screen Cover For Fiat Ducato Peugeot Boxer Citroen Relay RV Cover</t>
         </is>
       </c>
       <c r="H33" s="13" t="n"/>
@@ -2263,7 +2263,7 @@
       <c r="M33" s="14" t="n"/>
       <c r="N33" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005010318124054.html</t>
+          <t>https://www.aliexpress.com/item/1005011618553986.html</t>
         </is>
       </c>
       <c r="Q33" s="18" t="n"/>
@@ -2411,17 +2411,17 @@
     </row>
     <row r="37" ht="24" customHeight="1" s="71">
       <c r="A37" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Scbcc18495dd14007a943eb5d126f2372v.jpg")</f>
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sc87ec94ba4b94ae1b0f39ca26cfcad8dT.png")</f>
         <v/>
       </c>
       <c r="D37" s="18" t="inlineStr">
         <is>
-          <t>Downpipe Diverter Rectangular Shape Plastic Rainwater Diverter Downspo…</t>
+          <t>Solar Alarm IP65 Waterproof PIR Motion Detection Alarm with Siren and …</t>
         </is>
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $25.87. Vår räkning: landad ca 373 kr, tänkt butikspris 899 kr. Originaltitel: Downpipe Diverter Rectangular Shape Plastic Rainwater Diverter Downspout Rain Collector Corrugated Hose</t>
+          <t>AliExpress: US $23.07. Vår räkning: landad ca 332 kr, tänkt butikspris 799 kr. Originaltitel: Solar Alarm IP65 Waterproof PIR Motion Detection Alarm with Siren and Strobe Light For Home Security Alarm System</t>
         </is>
       </c>
       <c r="H37" s="13" t="n"/>
@@ -2436,7 +2436,7 @@
       <c r="M37" s="14" t="n"/>
       <c r="N37" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005012502051940.html</t>
+          <t>https://www.aliexpress.com/item/1005012241693262.html</t>
         </is>
       </c>
       <c r="Q37" s="18" t="n"/>
@@ -2582,179 +2582,10 @@
       <c r="AT40" s="35" t="n"/>
       <c r="AU40" s="35" t="n"/>
     </row>
-    <row r="41" ht="24" customHeight="1" s="71">
-      <c r="A41" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sc87ec94ba4b94ae1b0f39ca26cfcad8dT.png")</f>
-        <v/>
-      </c>
-      <c r="D41" s="18" t="inlineStr">
-        <is>
-          <t>Solar Alarm IP65 Waterproof PIR Motion Detection Alarm with Siren and …</t>
-        </is>
-      </c>
-      <c r="E41" s="12" t="inlineStr">
-        <is>
-          <t>AliExpress: US $23.07. Vår räkning: landad ca 332 kr, tänkt butikspris 799 kr. Originaltitel: Solar Alarm IP65 Waterproof PIR Motion Detection Alarm with Siren and Strobe Light For Home Security Alarm System</t>
-        </is>
-      </c>
-      <c r="H41" s="13" t="n"/>
-      <c r="I41" s="14" t="inlineStr">
-        <is>
-          <t>SWEDEN</t>
-        </is>
-      </c>
-      <c r="J41" s="15" t="n"/>
-      <c r="K41" s="15" t="n"/>
-      <c r="L41" s="16" t="n"/>
-      <c r="M41" s="14" t="n"/>
-      <c r="N41" s="17" t="inlineStr">
-        <is>
-          <t>https://www.aliexpress.com/item/1005012241693262.html</t>
-        </is>
-      </c>
-      <c r="Q41" s="18" t="n"/>
-      <c r="R41" s="19" t="n">
-        <v>100</v>
-      </c>
-      <c r="S41" s="15" t="n"/>
-      <c r="T41" s="15" t="n"/>
-      <c r="U41" s="16" t="n"/>
-      <c r="V41" s="48" t="n"/>
-      <c r="W41" s="48" t="n"/>
-      <c r="X41" s="21" t="n"/>
-      <c r="Y41" s="15" t="n"/>
-      <c r="Z41" s="15" t="n"/>
-      <c r="AA41" s="16" t="n"/>
-      <c r="AB41" s="48" t="n"/>
-      <c r="AC41" s="48" t="n"/>
-      <c r="AD41" s="22" t="n"/>
-      <c r="AE41" s="15" t="n"/>
-      <c r="AF41" s="15" t="n"/>
-      <c r="AG41" s="16" t="n"/>
-      <c r="AH41" s="48" t="n"/>
-      <c r="AI41" s="48" t="n"/>
-      <c r="AJ41" s="23" t="n"/>
-      <c r="AK41" s="15" t="n"/>
-      <c r="AL41" s="15" t="n"/>
-      <c r="AM41" s="16" t="n"/>
-      <c r="AN41" s="25" t="n"/>
-      <c r="AO41" s="48" t="n"/>
-      <c r="AP41" s="23" t="n"/>
-      <c r="AQ41" s="15" t="n"/>
-      <c r="AR41" s="15" t="n"/>
-      <c r="AS41" s="16" t="n"/>
-      <c r="AT41" s="25" t="n"/>
-      <c r="AU41" s="26" t="n"/>
-    </row>
-    <row r="42" ht="25.5" customHeight="1" s="71">
-      <c r="D42" s="18" t="n"/>
-      <c r="J42" s="15" t="n"/>
-      <c r="K42" s="15" t="n"/>
-      <c r="L42" s="16" t="n"/>
-      <c r="R42" s="19" t="n">
-        <v>200</v>
-      </c>
-      <c r="S42" s="15" t="n"/>
-      <c r="T42" s="15" t="n"/>
-      <c r="U42" s="16" t="n"/>
-      <c r="X42" s="21" t="n"/>
-      <c r="Y42" s="15" t="n"/>
-      <c r="Z42" s="15" t="n"/>
-      <c r="AA42" s="16" t="n"/>
-      <c r="AD42" s="22" t="n"/>
-      <c r="AE42" s="15" t="n"/>
-      <c r="AF42" s="15" t="n"/>
-      <c r="AG42" s="16" t="n"/>
-      <c r="AH42" s="48" t="n"/>
-      <c r="AI42" s="48" t="n"/>
-      <c r="AJ42" s="23" t="n"/>
-      <c r="AK42" s="15" t="n"/>
-      <c r="AL42" s="15" t="n"/>
-      <c r="AM42" s="16" t="n"/>
-      <c r="AP42" s="23" t="n"/>
-      <c r="AQ42" s="15" t="n"/>
-      <c r="AR42" s="15" t="n"/>
-      <c r="AS42" s="16" t="n"/>
-    </row>
-    <row r="43" s="71">
-      <c r="D43" s="18" t="n"/>
-      <c r="J43" s="15" t="n"/>
-      <c r="K43" s="15" t="n"/>
-      <c r="L43" s="16" t="n"/>
-      <c r="R43" s="19" t="n">
-        <v>300</v>
-      </c>
-      <c r="S43" s="15" t="n"/>
-      <c r="T43" s="15" t="n"/>
-      <c r="U43" s="16" t="n"/>
-      <c r="X43" s="21" t="n"/>
-      <c r="Y43" s="15" t="n"/>
-      <c r="Z43" s="15" t="n"/>
-      <c r="AA43" s="16" t="n"/>
-      <c r="AD43" s="22" t="n"/>
-      <c r="AE43" s="15" t="n"/>
-      <c r="AF43" s="15" t="n"/>
-      <c r="AG43" s="16" t="n"/>
-      <c r="AH43" s="48" t="n"/>
-      <c r="AI43" s="48" t="n"/>
-      <c r="AJ43" s="23" t="n"/>
-      <c r="AK43" s="15" t="n"/>
-      <c r="AL43" s="15" t="n"/>
-      <c r="AM43" s="16" t="n"/>
-      <c r="AP43" s="23" t="n"/>
-      <c r="AQ43" s="15" t="n"/>
-      <c r="AR43" s="15" t="n"/>
-      <c r="AS43" s="16" t="n"/>
-    </row>
-    <row r="44" ht="6.75" customHeight="1" s="71">
-      <c r="A44" s="27" t="n"/>
-      <c r="B44" s="27" t="n"/>
-      <c r="C44" s="27" t="n"/>
-      <c r="D44" s="27" t="n"/>
-      <c r="E44" s="27" t="n"/>
-      <c r="F44" s="27" t="n"/>
-      <c r="G44" s="27" t="n"/>
-      <c r="H44" s="35" t="n"/>
-      <c r="I44" s="35" t="n"/>
-      <c r="J44" s="36" t="n"/>
-      <c r="K44" s="36" t="n"/>
-      <c r="L44" s="36" t="n"/>
-      <c r="M44" s="35" t="n"/>
-      <c r="N44" s="30" t="n"/>
-      <c r="O44" s="30" t="n"/>
-      <c r="P44" s="30" t="n"/>
-      <c r="Q44" s="30" t="n"/>
-      <c r="R44" s="35" t="n"/>
-      <c r="S44" s="35" t="n"/>
-      <c r="T44" s="35" t="n"/>
-      <c r="U44" s="35" t="n"/>
-      <c r="V44" s="35" t="n"/>
-      <c r="W44" s="35" t="n"/>
-      <c r="X44" s="31" t="n"/>
-      <c r="Y44" s="35" t="n"/>
-      <c r="Z44" s="35" t="n"/>
-      <c r="AA44" s="36" t="n"/>
-      <c r="AB44" s="35" t="n"/>
-      <c r="AC44" s="35" t="n"/>
-      <c r="AD44" s="32" t="n"/>
-      <c r="AE44" s="35" t="n"/>
-      <c r="AF44" s="35" t="n"/>
-      <c r="AG44" s="36" t="n"/>
-      <c r="AH44" s="35" t="n"/>
-      <c r="AI44" s="35" t="n"/>
-      <c r="AJ44" s="34" t="n"/>
-      <c r="AK44" s="35" t="n"/>
-      <c r="AL44" s="35" t="n"/>
-      <c r="AM44" s="36" t="n"/>
-      <c r="AN44" s="35" t="n"/>
-      <c r="AO44" s="35" t="n"/>
-      <c r="AP44" s="34" t="n"/>
-      <c r="AQ44" s="35" t="n"/>
-      <c r="AR44" s="35" t="n"/>
-      <c r="AS44" s="36" t="n"/>
-      <c r="AT44" s="35" t="n"/>
-      <c r="AU44" s="35" t="n"/>
-    </row>
+    <row r="41" ht="15.75" customHeight="1" s="71"/>
+    <row r="42" ht="15.75" customHeight="1" s="71"/>
+    <row r="43" ht="15.75" customHeight="1" s="71"/>
+    <row r="44" ht="15.75" customHeight="1" s="71"/>
     <row r="45" ht="15.75" customHeight="1" s="71"/>
     <row r="46" ht="15.75" customHeight="1" s="71"/>
     <row r="47" ht="15.75" customHeight="1" s="71"/>
@@ -3712,19 +3543,17 @@
     <row r="999" ht="15.75" customHeight="1" s="71"/>
     <row r="1000" ht="15.75" customHeight="1" s="71"/>
   </sheetData>
-  <mergeCells count="87">
+  <mergeCells count="80">
     <mergeCell ref="E5:G7"/>
     <mergeCell ref="H17:H19"/>
     <mergeCell ref="M21:M23"/>
     <mergeCell ref="L3:L4"/>
     <mergeCell ref="N5:P7"/>
-    <mergeCell ref="M41:M43"/>
     <mergeCell ref="N33:P35"/>
     <mergeCell ref="A37:C39"/>
     <mergeCell ref="R3:W3"/>
     <mergeCell ref="A21:C23"/>
     <mergeCell ref="I3:I4"/>
-    <mergeCell ref="Q41:Q43"/>
     <mergeCell ref="H5:H7"/>
     <mergeCell ref="A29:C31"/>
     <mergeCell ref="M5:M7"/>
@@ -3750,14 +3579,12 @@
     <mergeCell ref="N3:P4"/>
     <mergeCell ref="H25:H27"/>
     <mergeCell ref="N9:P11"/>
-    <mergeCell ref="I41:I43"/>
     <mergeCell ref="E21:G23"/>
     <mergeCell ref="K3:K4"/>
     <mergeCell ref="I25:I27"/>
     <mergeCell ref="I33:I35"/>
     <mergeCell ref="I5:I7"/>
     <mergeCell ref="I17:I19"/>
-    <mergeCell ref="A41:C43"/>
     <mergeCell ref="N37:P39"/>
     <mergeCell ref="X3:AC3"/>
     <mergeCell ref="M33:M35"/>
@@ -3780,7 +3607,6 @@
     <mergeCell ref="J3:J4"/>
     <mergeCell ref="H9:H11"/>
     <mergeCell ref="E37:G39"/>
-    <mergeCell ref="N41:P43"/>
     <mergeCell ref="N25:P27"/>
     <mergeCell ref="M13:M15"/>
     <mergeCell ref="E29:G31"/>
@@ -3790,9 +3616,7 @@
     <mergeCell ref="N29:P31"/>
     <mergeCell ref="I9:I11"/>
     <mergeCell ref="A33:C35"/>
-    <mergeCell ref="E41:G43"/>
     <mergeCell ref="A3:C4"/>
-    <mergeCell ref="H41:H43"/>
     <mergeCell ref="Q5:Q7"/>
     <mergeCell ref="A2:AO2"/>
     <mergeCell ref="E33:G35"/>

</xml_diff>

<commit_message>
produktjakt: sasongen bedoms mot halvan av manaden, inte manadsnumret
Axels papekande 2026-09-09: vi ar i MITTEN av september. Da tas batarna upp,
sa ett navigationsljus (Solar Marine Signal Lights) ar utrustning for nasta
sasong, inte for nu. Struket ur dagens leverans — 8 produkter kvar av 22
granskade — och sokordet flyttat till nya gruppen "var och forsasong" (manad
4-6) tillsammans med regnvattenavledaren.

Regeln star nu i kommandots steg 2: avstallning och skydd saljs nu,
utrustning som ska anvandas nasta sasong hor hemma i april-juni.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016jBJVGuyny8S3j2XPSM26Z
</commit_message>
<xml_diff>
--- a/produktjakt/korningar/2026-09-09/Leverantorsoffert-2026-09-09.xlsx
+++ b/produktjakt/korningar/2026-09-09/Leverantorsoffert-2026-09-09.xlsx
@@ -732,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU40"/>
+  <dimension ref="A1:AU36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="18" customWidth="1" style="71" min="1" max="1"/>
@@ -767,7 +767,7 @@
   <sheetData>
     <row r="1" ht="27.75" customHeight="1" s="71">
       <c r="A1" s="1" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AP1" s="1" t="n"/>
       <c r="AQ1" s="1" t="n"/>
@@ -2065,17 +2065,17 @@
     </row>
     <row r="29" ht="24" customHeight="1" s="71">
       <c r="A29" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S4244c19ccbb7400787c5f68f47dda6f9q.jpg")</f>
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sd45dbbc9fcb64ef4a78670e4fe959d40T.png")</f>
         <v/>
       </c>
       <c r="D29" s="18" t="inlineStr">
         <is>
-          <t>Solar Powered Marine Signal Lights LED Navigation Warning Lamps Waterp…</t>
+          <t>Windshield Sunshade Front Motorhome Thermal Windscreen Screen Cover Fo…</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $11.00. Vår räkning: landad ca 158 kr, tänkt butikspris 399 kr. Originaltitel: Solar Powered Marine Signal Lights LED Navigation Warning Lamps Waterproof Boat Marker Beacons For Yacht Fishing Vessel</t>
+          <t>AliExpress: US $19.67. Vår räkning: landad ca 283 kr, tänkt butikspris 699 kr. Originaltitel: Windshield Sunshade Front Motorhome Thermal Windscreen Screen Cover For Fiat Ducato Peugeot Boxer Citroen Relay RV Cover</t>
         </is>
       </c>
       <c r="H29" s="13" t="n"/>
@@ -2090,7 +2090,7 @@
       <c r="M29" s="14" t="n"/>
       <c r="N29" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005011767102250.html</t>
+          <t>https://www.aliexpress.com/item/1005011618553986.html</t>
         </is>
       </c>
       <c r="Q29" s="18" t="n"/>
@@ -2238,17 +2238,17 @@
     </row>
     <row r="33" ht="24" customHeight="1" s="71">
       <c r="A33" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sd45dbbc9fcb64ef4a78670e4fe959d40T.png")</f>
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sc87ec94ba4b94ae1b0f39ca26cfcad8dT.png")</f>
         <v/>
       </c>
       <c r="D33" s="18" t="inlineStr">
         <is>
-          <t>Windshield Sunshade Front Motorhome Thermal Windscreen Screen Cover Fo…</t>
+          <t>Solar Alarm IP65 Waterproof PIR Motion Detection Alarm with Siren and …</t>
         </is>
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $19.67. Vår räkning: landad ca 283 kr, tänkt butikspris 699 kr. Originaltitel: Windshield Sunshade Front Motorhome Thermal Windscreen Screen Cover For Fiat Ducato Peugeot Boxer Citroen Relay RV Cover</t>
+          <t>AliExpress: US $23.07. Vår räkning: landad ca 332 kr, tänkt butikspris 799 kr. Originaltitel: Solar Alarm IP65 Waterproof PIR Motion Detection Alarm with Siren and Strobe Light For Home Security Alarm System</t>
         </is>
       </c>
       <c r="H33" s="13" t="n"/>
@@ -2263,7 +2263,7 @@
       <c r="M33" s="14" t="n"/>
       <c r="N33" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005011618553986.html</t>
+          <t>https://www.aliexpress.com/item/1005012241693262.html</t>
         </is>
       </c>
       <c r="Q33" s="18" t="n"/>
@@ -2409,179 +2409,10 @@
       <c r="AT36" s="35" t="n"/>
       <c r="AU36" s="35" t="n"/>
     </row>
-    <row r="37" ht="24" customHeight="1" s="71">
-      <c r="A37" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sc87ec94ba4b94ae1b0f39ca26cfcad8dT.png")</f>
-        <v/>
-      </c>
-      <c r="D37" s="18" t="inlineStr">
-        <is>
-          <t>Solar Alarm IP65 Waterproof PIR Motion Detection Alarm with Siren and …</t>
-        </is>
-      </c>
-      <c r="E37" s="12" t="inlineStr">
-        <is>
-          <t>AliExpress: US $23.07. Vår räkning: landad ca 332 kr, tänkt butikspris 799 kr. Originaltitel: Solar Alarm IP65 Waterproof PIR Motion Detection Alarm with Siren and Strobe Light For Home Security Alarm System</t>
-        </is>
-      </c>
-      <c r="H37" s="13" t="n"/>
-      <c r="I37" s="14" t="inlineStr">
-        <is>
-          <t>SWEDEN</t>
-        </is>
-      </c>
-      <c r="J37" s="15" t="n"/>
-      <c r="K37" s="15" t="n"/>
-      <c r="L37" s="16" t="n"/>
-      <c r="M37" s="14" t="n"/>
-      <c r="N37" s="17" t="inlineStr">
-        <is>
-          <t>https://www.aliexpress.com/item/1005012241693262.html</t>
-        </is>
-      </c>
-      <c r="Q37" s="18" t="n"/>
-      <c r="R37" s="19" t="n">
-        <v>100</v>
-      </c>
-      <c r="S37" s="15" t="n"/>
-      <c r="T37" s="15" t="n"/>
-      <c r="U37" s="16" t="n"/>
-      <c r="V37" s="48" t="n"/>
-      <c r="W37" s="48" t="n"/>
-      <c r="X37" s="21" t="n"/>
-      <c r="Y37" s="15" t="n"/>
-      <c r="Z37" s="15" t="n"/>
-      <c r="AA37" s="16" t="n"/>
-      <c r="AB37" s="48" t="n"/>
-      <c r="AC37" s="48" t="n"/>
-      <c r="AD37" s="22" t="n"/>
-      <c r="AE37" s="15" t="n"/>
-      <c r="AF37" s="15" t="n"/>
-      <c r="AG37" s="16" t="n"/>
-      <c r="AH37" s="48" t="n"/>
-      <c r="AI37" s="48" t="n"/>
-      <c r="AJ37" s="23" t="n"/>
-      <c r="AK37" s="15" t="n"/>
-      <c r="AL37" s="15" t="n"/>
-      <c r="AM37" s="16" t="n"/>
-      <c r="AN37" s="25" t="n"/>
-      <c r="AO37" s="48" t="n"/>
-      <c r="AP37" s="23" t="n"/>
-      <c r="AQ37" s="15" t="n"/>
-      <c r="AR37" s="15" t="n"/>
-      <c r="AS37" s="16" t="n"/>
-      <c r="AT37" s="25" t="n"/>
-      <c r="AU37" s="26" t="n"/>
-    </row>
-    <row r="38" ht="25.5" customHeight="1" s="71">
-      <c r="D38" s="18" t="n"/>
-      <c r="J38" s="15" t="n"/>
-      <c r="K38" s="15" t="n"/>
-      <c r="L38" s="16" t="n"/>
-      <c r="R38" s="19" t="n">
-        <v>200</v>
-      </c>
-      <c r="S38" s="15" t="n"/>
-      <c r="T38" s="15" t="n"/>
-      <c r="U38" s="16" t="n"/>
-      <c r="X38" s="21" t="n"/>
-      <c r="Y38" s="15" t="n"/>
-      <c r="Z38" s="15" t="n"/>
-      <c r="AA38" s="16" t="n"/>
-      <c r="AD38" s="22" t="n"/>
-      <c r="AE38" s="15" t="n"/>
-      <c r="AF38" s="15" t="n"/>
-      <c r="AG38" s="16" t="n"/>
-      <c r="AH38" s="48" t="n"/>
-      <c r="AI38" s="48" t="n"/>
-      <c r="AJ38" s="23" t="n"/>
-      <c r="AK38" s="15" t="n"/>
-      <c r="AL38" s="15" t="n"/>
-      <c r="AM38" s="16" t="n"/>
-      <c r="AP38" s="23" t="n"/>
-      <c r="AQ38" s="15" t="n"/>
-      <c r="AR38" s="15" t="n"/>
-      <c r="AS38" s="16" t="n"/>
-    </row>
-    <row r="39" s="71">
-      <c r="D39" s="18" t="n"/>
-      <c r="J39" s="15" t="n"/>
-      <c r="K39" s="15" t="n"/>
-      <c r="L39" s="16" t="n"/>
-      <c r="R39" s="19" t="n">
-        <v>300</v>
-      </c>
-      <c r="S39" s="15" t="n"/>
-      <c r="T39" s="15" t="n"/>
-      <c r="U39" s="16" t="n"/>
-      <c r="X39" s="21" t="n"/>
-      <c r="Y39" s="15" t="n"/>
-      <c r="Z39" s="15" t="n"/>
-      <c r="AA39" s="16" t="n"/>
-      <c r="AD39" s="22" t="n"/>
-      <c r="AE39" s="15" t="n"/>
-      <c r="AF39" s="15" t="n"/>
-      <c r="AG39" s="16" t="n"/>
-      <c r="AH39" s="48" t="n"/>
-      <c r="AI39" s="48" t="n"/>
-      <c r="AJ39" s="23" t="n"/>
-      <c r="AK39" s="15" t="n"/>
-      <c r="AL39" s="15" t="n"/>
-      <c r="AM39" s="16" t="n"/>
-      <c r="AP39" s="23" t="n"/>
-      <c r="AQ39" s="15" t="n"/>
-      <c r="AR39" s="15" t="n"/>
-      <c r="AS39" s="16" t="n"/>
-    </row>
-    <row r="40" ht="6.75" customHeight="1" s="71">
-      <c r="A40" s="27" t="n"/>
-      <c r="B40" s="27" t="n"/>
-      <c r="C40" s="27" t="n"/>
-      <c r="D40" s="27" t="n"/>
-      <c r="E40" s="27" t="n"/>
-      <c r="F40" s="27" t="n"/>
-      <c r="G40" s="27" t="n"/>
-      <c r="H40" s="35" t="n"/>
-      <c r="I40" s="35" t="n"/>
-      <c r="J40" s="36" t="n"/>
-      <c r="K40" s="36" t="n"/>
-      <c r="L40" s="36" t="n"/>
-      <c r="M40" s="35" t="n"/>
-      <c r="N40" s="30" t="n"/>
-      <c r="O40" s="30" t="n"/>
-      <c r="P40" s="30" t="n"/>
-      <c r="Q40" s="30" t="n"/>
-      <c r="R40" s="35" t="n"/>
-      <c r="S40" s="35" t="n"/>
-      <c r="T40" s="35" t="n"/>
-      <c r="U40" s="35" t="n"/>
-      <c r="V40" s="35" t="n"/>
-      <c r="W40" s="35" t="n"/>
-      <c r="X40" s="31" t="n"/>
-      <c r="Y40" s="35" t="n"/>
-      <c r="Z40" s="35" t="n"/>
-      <c r="AA40" s="36" t="n"/>
-      <c r="AB40" s="35" t="n"/>
-      <c r="AC40" s="35" t="n"/>
-      <c r="AD40" s="32" t="n"/>
-      <c r="AE40" s="35" t="n"/>
-      <c r="AF40" s="35" t="n"/>
-      <c r="AG40" s="36" t="n"/>
-      <c r="AH40" s="35" t="n"/>
-      <c r="AI40" s="35" t="n"/>
-      <c r="AJ40" s="34" t="n"/>
-      <c r="AK40" s="35" t="n"/>
-      <c r="AL40" s="35" t="n"/>
-      <c r="AM40" s="36" t="n"/>
-      <c r="AN40" s="35" t="n"/>
-      <c r="AO40" s="35" t="n"/>
-      <c r="AP40" s="34" t="n"/>
-      <c r="AQ40" s="35" t="n"/>
-      <c r="AR40" s="35" t="n"/>
-      <c r="AS40" s="36" t="n"/>
-      <c r="AT40" s="35" t="n"/>
-      <c r="AU40" s="35" t="n"/>
-    </row>
+    <row r="37" ht="15.75" customHeight="1" s="71"/>
+    <row r="38" ht="15.75" customHeight="1" s="71"/>
+    <row r="39" ht="15.75" customHeight="1" s="71"/>
+    <row r="40" ht="15.75" customHeight="1" s="71"/>
     <row r="41" ht="15.75" customHeight="1" s="71"/>
     <row r="42" ht="15.75" customHeight="1" s="71"/>
     <row r="43" ht="15.75" customHeight="1" s="71"/>
@@ -3543,87 +3374,80 @@
     <row r="999" ht="15.75" customHeight="1" s="71"/>
     <row r="1000" ht="15.75" customHeight="1" s="71"/>
   </sheetData>
-  <mergeCells count="80">
+  <mergeCells count="73">
+    <mergeCell ref="I5:I7"/>
     <mergeCell ref="E5:G7"/>
+    <mergeCell ref="Q9:Q11"/>
     <mergeCell ref="H17:H19"/>
+    <mergeCell ref="I17:I19"/>
     <mergeCell ref="M21:M23"/>
     <mergeCell ref="L3:L4"/>
-    <mergeCell ref="N5:P7"/>
-    <mergeCell ref="N33:P35"/>
-    <mergeCell ref="A37:C39"/>
-    <mergeCell ref="R3:W3"/>
-    <mergeCell ref="A21:C23"/>
-    <mergeCell ref="I3:I4"/>
-    <mergeCell ref="H5:H7"/>
-    <mergeCell ref="A29:C31"/>
-    <mergeCell ref="M5:M7"/>
-    <mergeCell ref="H29:H31"/>
-    <mergeCell ref="A13:C15"/>
-    <mergeCell ref="Q33:Q35"/>
-    <mergeCell ref="AD3:AI3"/>
-    <mergeCell ref="E25:G27"/>
-    <mergeCell ref="AP3:AU3"/>
-    <mergeCell ref="H21:H23"/>
-    <mergeCell ref="M25:M27"/>
-    <mergeCell ref="Q3:Q4"/>
-    <mergeCell ref="E17:G19"/>
-    <mergeCell ref="I37:I39"/>
-    <mergeCell ref="Q9:Q11"/>
-    <mergeCell ref="I29:I31"/>
-    <mergeCell ref="I13:I15"/>
-    <mergeCell ref="M29:M31"/>
-    <mergeCell ref="A1:AO1"/>
-    <mergeCell ref="H33:H35"/>
-    <mergeCell ref="N17:P19"/>
-    <mergeCell ref="A5:C7"/>
-    <mergeCell ref="N3:P4"/>
-    <mergeCell ref="H25:H27"/>
-    <mergeCell ref="N9:P11"/>
-    <mergeCell ref="E21:G23"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="I25:I27"/>
-    <mergeCell ref="I33:I35"/>
-    <mergeCell ref="I5:I7"/>
-    <mergeCell ref="I17:I19"/>
-    <mergeCell ref="N37:P39"/>
+    <mergeCell ref="E13:G15"/>
     <mergeCell ref="X3:AC3"/>
     <mergeCell ref="M33:M35"/>
     <mergeCell ref="N21:P23"/>
+    <mergeCell ref="I29:I31"/>
+    <mergeCell ref="N5:P7"/>
     <mergeCell ref="H13:H15"/>
     <mergeCell ref="E3:G4"/>
     <mergeCell ref="A25:C27"/>
     <mergeCell ref="AJ3:AO3"/>
+    <mergeCell ref="N33:P35"/>
     <mergeCell ref="M17:M19"/>
+    <mergeCell ref="I13:I15"/>
     <mergeCell ref="Q17:Q19"/>
     <mergeCell ref="E9:G11"/>
+    <mergeCell ref="R3:W3"/>
+    <mergeCell ref="A21:C23"/>
+    <mergeCell ref="M29:M31"/>
+    <mergeCell ref="A1:AO1"/>
     <mergeCell ref="M3:M4"/>
+    <mergeCell ref="I3:I4"/>
     <mergeCell ref="Q13:Q15"/>
     <mergeCell ref="N13:P15"/>
+    <mergeCell ref="N17:P19"/>
+    <mergeCell ref="Q25:Q27"/>
     <mergeCell ref="A17:C19"/>
-    <mergeCell ref="M9:M11"/>
-    <mergeCell ref="Q37:Q39"/>
-    <mergeCell ref="Q21:Q23"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="J3:J4"/>
-    <mergeCell ref="H9:H11"/>
-    <mergeCell ref="E37:G39"/>
-    <mergeCell ref="N25:P27"/>
-    <mergeCell ref="M13:M15"/>
-    <mergeCell ref="E29:G31"/>
-    <mergeCell ref="E13:G15"/>
-    <mergeCell ref="H37:H39"/>
-    <mergeCell ref="Q25:Q27"/>
+    <mergeCell ref="H33:H35"/>
+    <mergeCell ref="H5:H7"/>
     <mergeCell ref="N29:P31"/>
     <mergeCell ref="I9:I11"/>
     <mergeCell ref="A33:C35"/>
+    <mergeCell ref="A29:C31"/>
+    <mergeCell ref="A5:C7"/>
+    <mergeCell ref="N3:P4"/>
+    <mergeCell ref="M9:M11"/>
+    <mergeCell ref="M5:M7"/>
+    <mergeCell ref="H29:H31"/>
+    <mergeCell ref="A13:C15"/>
+    <mergeCell ref="Q21:Q23"/>
+    <mergeCell ref="H25:H27"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="N9:P11"/>
+    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="Q33:Q35"/>
     <mergeCell ref="A3:C4"/>
+    <mergeCell ref="AD3:AI3"/>
+    <mergeCell ref="E25:G27"/>
+    <mergeCell ref="E21:G23"/>
     <mergeCell ref="Q5:Q7"/>
+    <mergeCell ref="AP3:AU3"/>
+    <mergeCell ref="H9:H11"/>
     <mergeCell ref="A2:AO2"/>
     <mergeCell ref="E33:G35"/>
+    <mergeCell ref="K3:K4"/>
     <mergeCell ref="A9:C11"/>
+    <mergeCell ref="H21:H23"/>
+    <mergeCell ref="I25:I27"/>
+    <mergeCell ref="M25:M27"/>
+    <mergeCell ref="Q3:Q4"/>
     <mergeCell ref="Q29:Q31"/>
     <mergeCell ref="I21:I23"/>
-    <mergeCell ref="M37:M39"/>
+    <mergeCell ref="E17:G19"/>
+    <mergeCell ref="N25:P27"/>
+    <mergeCell ref="I33:I35"/>
+    <mergeCell ref="M13:M15"/>
+    <mergeCell ref="E29:G31"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId1"/>

</xml_diff>

<commit_message>
produktjakt: jamfor mot forra arket pa produkt, inte pa id
Axel kande igen fyra av atta varor fran gardagens ark: sittkappen,
stegstabilisatorn, vindrutekapan och solcellslarmet. Alla fyra strukna.

Tva orsaker. Gardagens jakt lag i docs/temu-jakt-v2/jakt/v24/ och dess sex
produkter kom aldrig in i sedda.json — de ar inlagda nu. Och id-jamforelsen
racker inte: samma vara saljs av flera saljare med olika product_id, sa
lasningen maste jamfora mot forra korningens lista pa produkt. Det star nu
som eget stryk-kriterium i kommandots steg 2.

En tredje sokomgang kordes for att ersatta de strukna. Dagens leverans ar
5 varor av 43 granskade, ingen av dem pa gardagens ark.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016jBJVGuyny8S3j2XPSM26Z
</commit_message>
<xml_diff>
--- a/produktjakt/korningar/2026-09-09/Leverantorsoffert-2026-09-09.xlsx
+++ b/produktjakt/korningar/2026-09-09/Leverantorsoffert-2026-09-09.xlsx
@@ -732,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU36"/>
+  <dimension ref="A1:AU24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="18" customWidth="1" style="71" min="1" max="1"/>
@@ -767,7 +767,7 @@
   <sheetData>
     <row r="1" ht="27.75" customHeight="1" s="71">
       <c r="A1" s="1" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="AP1" s="1" t="n"/>
       <c r="AQ1" s="1" t="n"/>
@@ -1200,17 +1200,17 @@
     </row>
     <row r="9" ht="24" customHeight="1" s="71">
       <c r="A9" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sddf296c4c78d43d7a1d84ca5614acb6fL.jpg")</f>
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S20416daaf99f4237ab753083a39afac5H.jpg")</f>
         <v/>
       </c>
       <c r="D9" s="18" t="inlineStr">
         <is>
-          <t>Foldable Cane Easy To Carry Seat Portable Stool Folding Chair Non Slip…</t>
+          <t>Winter Warm Waterproof Stray Cat Dog House Foldable Washable Pet Cave …</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $16.08. Vår räkning: landad ca 232 kr, tänkt butikspris 599 kr. Originaltitel: Foldable Cane Easy To Carry Seat Portable Stool Folding Chair Non Slip Handle Super Light Walking Stick For Outdoor Walking</t>
+          <t>AliExpress: US $21.66. Vår räkning: landad ca 312 kr, tänkt butikspris 799 kr. Originaltitel: Winter Warm Waterproof Stray Cat Dog House Foldable Washable Pet Cave Outdoor Shelter Sleeping Bed for Small Puppy Pet Supplies</t>
         </is>
       </c>
       <c r="H9" s="13" t="n"/>
@@ -1225,7 +1225,7 @@
       <c r="M9" s="14" t="n"/>
       <c r="N9" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005011927514185.html</t>
+          <t>https://www.aliexpress.com/item/1005012414077421.html</t>
         </is>
       </c>
       <c r="Q9" s="18" t="n"/>
@@ -1373,17 +1373,17 @@
     </row>
     <row r="13" ht="24" customHeight="1" s="71">
       <c r="A13" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S20416daaf99f4237ab753083a39afac5H.jpg")</f>
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sf82b0d4f34464eaca317489c4e31f25f8.jpg")</f>
         <v/>
       </c>
       <c r="D13" s="18" t="inlineStr">
         <is>
-          <t>Winter Warm Waterproof Stray Cat Dog House Foldable Washable Pet Cave …</t>
+          <t>Professional Telescopic Boat Cover Support Pole Windproof Adjustable H…</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $21.66. Vår räkning: landad ca 312 kr, tänkt butikspris 799 kr. Originaltitel: Winter Warm Waterproof Stray Cat Dog House Foldable Washable Pet Cave Outdoor Shelter Sleeping Bed for Small Puppy Pet Supplies</t>
+          <t>AliExpress: US $10.77. Vår räkning: landad ca 155 kr, tänkt butikspris 399 kr. Originaltitel: Professional Telescopic Boat Cover Support Pole Windproof Adjustable Height 22"-70" Heavy-Duty Steel/Aluminum for Pontoon Patio</t>
         </is>
       </c>
       <c r="H13" s="13" t="n"/>
@@ -1398,7 +1398,7 @@
       <c r="M13" s="14" t="n"/>
       <c r="N13" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005012414077421.html</t>
+          <t>https://www.aliexpress.com/item/1005009100129778.html</t>
         </is>
       </c>
       <c r="Q13" s="18" t="n"/>
@@ -1546,17 +1546,17 @@
     </row>
     <row r="17" ht="24" customHeight="1" s="71">
       <c r="A17" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sf82b0d4f34464eaca317489c4e31f25f8.jpg")</f>
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S1765e6b203364ba5b2b27145c16238989.jpg")</f>
         <v/>
       </c>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>Professional Telescopic Boat Cover Support Pole Windproof Adjustable H…</t>
+          <t>Outboard Motor Flusher Muffs Kit with 16mm Quick Connect Fitting, Adju…</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $10.77. Vår räkning: landad ca 155 kr, tänkt butikspris 399 kr. Originaltitel: Professional Telescopic Boat Cover Support Pole Windproof Adjustable Height 22"-70" Heavy-Duty Steel/Aluminum for Pontoon Patio</t>
+          <t>AliExpress: US $25.05. Vår räkning: landad ca 361 kr, tänkt butikspris 899 kr. Originaltitel: Outboard Motor Flusher Muffs Kit with 16mm Quick Connect Fitting, Adjustable Dual/Single Tube for Boat Motor Cleaning &amp; Test Run</t>
         </is>
       </c>
       <c r="H17" s="13" t="n"/>
@@ -1571,7 +1571,7 @@
       <c r="M17" s="14" t="n"/>
       <c r="N17" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005009100129778.html</t>
+          <t>https://www.aliexpress.com/item/1005011764722846.html</t>
         </is>
       </c>
       <c r="Q17" s="18" t="n"/>
@@ -1719,17 +1719,17 @@
     </row>
     <row r="21" ht="24" customHeight="1" s="71">
       <c r="A21" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S1765e6b203364ba5b2b27145c16238989.jpg")</f>
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sda69235967df40a5a5442b5e4f1323c5M.jpg")</f>
         <v/>
       </c>
       <c r="D21" s="18" t="inlineStr">
         <is>
-          <t>Outboard Motor Flusher Muffs Kit with 16mm Quick Connect Fitting, Adju…</t>
+          <t>1/2 Pack Heavy Duty Steel Fence Post Repair Kit - Anchor Brackets &amp; Gr…</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $25.05. Vår räkning: landad ca 361 kr, tänkt butikspris 899 kr. Originaltitel: Outboard Motor Flusher Muffs Kit with 16mm Quick Connect Fitting, Adjustable Dual/Single Tube for Boat Motor Cleaning &amp; Test Run</t>
+          <t>AliExpress: US $18.74. Vår räkning: landad ca 270 kr, tänkt butikspris 699 kr. Originaltitel: 1/2 Pack Heavy Duty Steel Fence Post Repair Kit - Anchor Brackets &amp; Ground Spike for Fixing Tilted/Broken Wooden Fence Posts</t>
         </is>
       </c>
       <c r="H21" s="13" t="n"/>
@@ -1744,7 +1744,7 @@
       <c r="M21" s="14" t="n"/>
       <c r="N21" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005011764722846.html</t>
+          <t>https://www.aliexpress.com/item/1005009145737438.html</t>
         </is>
       </c>
       <c r="Q21" s="18" t="n"/>
@@ -1890,525 +1890,18 @@
       <c r="AT24" s="35" t="n"/>
       <c r="AU24" s="35" t="n"/>
     </row>
-    <row r="25" ht="24" customHeight="1" s="71">
-      <c r="A25" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S4f5c23377f414f0c868c1af6496a8f73E.jpg")</f>
-        <v/>
-      </c>
-      <c r="D25" s="18" t="inlineStr">
-        <is>
-          <t>Roof Ladder Stabilizer, Ladder Standoff, Extension Ladder Stabilizer, …</t>
-        </is>
-      </c>
-      <c r="E25" s="12" t="inlineStr">
-        <is>
-          <t>AliExpress: US $27.55. Vår räkning: landad ca 397 kr, tänkt butikspris 999 kr. Originaltitel: Roof Ladder Stabilizer, Ladder Standoff, Extension Ladder Stabilizer, Wall Bracket, Heavy Duty Secure</t>
-        </is>
-      </c>
-      <c r="H25" s="13" t="n"/>
-      <c r="I25" s="14" t="inlineStr">
-        <is>
-          <t>SWEDEN</t>
-        </is>
-      </c>
-      <c r="J25" s="15" t="n"/>
-      <c r="K25" s="15" t="n"/>
-      <c r="L25" s="16" t="n"/>
-      <c r="M25" s="14" t="n"/>
-      <c r="N25" s="17" t="inlineStr">
-        <is>
-          <t>https://www.aliexpress.com/item/1005012386302696.html</t>
-        </is>
-      </c>
-      <c r="Q25" s="18" t="n"/>
-      <c r="R25" s="19" t="n">
-        <v>100</v>
-      </c>
-      <c r="S25" s="15" t="n"/>
-      <c r="T25" s="15" t="n"/>
-      <c r="U25" s="16" t="n"/>
-      <c r="V25" s="48" t="n"/>
-      <c r="W25" s="48" t="n"/>
-      <c r="X25" s="21" t="n"/>
-      <c r="Y25" s="15" t="n"/>
-      <c r="Z25" s="15" t="n"/>
-      <c r="AA25" s="16" t="n"/>
-      <c r="AB25" s="48" t="n"/>
-      <c r="AC25" s="48" t="n"/>
-      <c r="AD25" s="22" t="n"/>
-      <c r="AE25" s="15" t="n"/>
-      <c r="AF25" s="15" t="n"/>
-      <c r="AG25" s="16" t="n"/>
-      <c r="AH25" s="48" t="n"/>
-      <c r="AI25" s="48" t="n"/>
-      <c r="AJ25" s="23" t="n"/>
-      <c r="AK25" s="15" t="n"/>
-      <c r="AL25" s="15" t="n"/>
-      <c r="AM25" s="16" t="n"/>
-      <c r="AN25" s="25" t="n"/>
-      <c r="AO25" s="48" t="n"/>
-      <c r="AP25" s="23" t="n"/>
-      <c r="AQ25" s="15" t="n"/>
-      <c r="AR25" s="15" t="n"/>
-      <c r="AS25" s="16" t="n"/>
-      <c r="AT25" s="25" t="n"/>
-      <c r="AU25" s="26" t="n"/>
-    </row>
-    <row r="26" ht="25.5" customHeight="1" s="71">
-      <c r="D26" s="18" t="n"/>
-      <c r="J26" s="15" t="n"/>
-      <c r="K26" s="15" t="n"/>
-      <c r="L26" s="16" t="n"/>
-      <c r="R26" s="19" t="n">
-        <v>200</v>
-      </c>
-      <c r="S26" s="15" t="n"/>
-      <c r="T26" s="15" t="n"/>
-      <c r="U26" s="16" t="n"/>
-      <c r="X26" s="21" t="n"/>
-      <c r="Y26" s="15" t="n"/>
-      <c r="Z26" s="15" t="n"/>
-      <c r="AA26" s="16" t="n"/>
-      <c r="AD26" s="22" t="n"/>
-      <c r="AE26" s="15" t="n"/>
-      <c r="AF26" s="15" t="n"/>
-      <c r="AG26" s="16" t="n"/>
-      <c r="AH26" s="48" t="n"/>
-      <c r="AI26" s="48" t="n"/>
-      <c r="AJ26" s="23" t="n"/>
-      <c r="AK26" s="15" t="n"/>
-      <c r="AL26" s="15" t="n"/>
-      <c r="AM26" s="16" t="n"/>
-      <c r="AP26" s="23" t="n"/>
-      <c r="AQ26" s="15" t="n"/>
-      <c r="AR26" s="15" t="n"/>
-      <c r="AS26" s="16" t="n"/>
-    </row>
-    <row r="27" s="71">
-      <c r="D27" s="18" t="n"/>
-      <c r="J27" s="15" t="n"/>
-      <c r="K27" s="15" t="n"/>
-      <c r="L27" s="16" t="n"/>
-      <c r="R27" s="19" t="n">
-        <v>300</v>
-      </c>
-      <c r="S27" s="15" t="n"/>
-      <c r="T27" s="15" t="n"/>
-      <c r="U27" s="16" t="n"/>
-      <c r="X27" s="21" t="n"/>
-      <c r="Y27" s="15" t="n"/>
-      <c r="Z27" s="15" t="n"/>
-      <c r="AA27" s="16" t="n"/>
-      <c r="AD27" s="22" t="n"/>
-      <c r="AE27" s="15" t="n"/>
-      <c r="AF27" s="15" t="n"/>
-      <c r="AG27" s="16" t="n"/>
-      <c r="AH27" s="48" t="n"/>
-      <c r="AI27" s="48" t="n"/>
-      <c r="AJ27" s="23" t="n"/>
-      <c r="AK27" s="15" t="n"/>
-      <c r="AL27" s="15" t="n"/>
-      <c r="AM27" s="16" t="n"/>
-      <c r="AP27" s="23" t="n"/>
-      <c r="AQ27" s="15" t="n"/>
-      <c r="AR27" s="15" t="n"/>
-      <c r="AS27" s="16" t="n"/>
-    </row>
-    <row r="28" ht="6.75" customHeight="1" s="71">
-      <c r="A28" s="27" t="n"/>
-      <c r="B28" s="27" t="n"/>
-      <c r="C28" s="27" t="n"/>
-      <c r="D28" s="27" t="n"/>
-      <c r="E28" s="27" t="n"/>
-      <c r="F28" s="27" t="n"/>
-      <c r="G28" s="27" t="n"/>
-      <c r="H28" s="35" t="n"/>
-      <c r="I28" s="35" t="n"/>
-      <c r="J28" s="36" t="n"/>
-      <c r="K28" s="36" t="n"/>
-      <c r="L28" s="36" t="n"/>
-      <c r="M28" s="35" t="n"/>
-      <c r="N28" s="30" t="n"/>
-      <c r="O28" s="30" t="n"/>
-      <c r="P28" s="30" t="n"/>
-      <c r="Q28" s="30" t="n"/>
-      <c r="R28" s="35" t="n"/>
-      <c r="S28" s="35" t="n"/>
-      <c r="T28" s="35" t="n"/>
-      <c r="U28" s="35" t="n"/>
-      <c r="V28" s="35" t="n"/>
-      <c r="W28" s="35" t="n"/>
-      <c r="X28" s="31" t="n"/>
-      <c r="Y28" s="35" t="n"/>
-      <c r="Z28" s="35" t="n"/>
-      <c r="AA28" s="36" t="n"/>
-      <c r="AB28" s="35" t="n"/>
-      <c r="AC28" s="35" t="n"/>
-      <c r="AD28" s="32" t="n"/>
-      <c r="AE28" s="35" t="n"/>
-      <c r="AF28" s="35" t="n"/>
-      <c r="AG28" s="36" t="n"/>
-      <c r="AH28" s="35" t="n"/>
-      <c r="AI28" s="35" t="n"/>
-      <c r="AJ28" s="34" t="n"/>
-      <c r="AK28" s="35" t="n"/>
-      <c r="AL28" s="35" t="n"/>
-      <c r="AM28" s="36" t="n"/>
-      <c r="AN28" s="35" t="n"/>
-      <c r="AO28" s="35" t="n"/>
-      <c r="AP28" s="34" t="n"/>
-      <c r="AQ28" s="35" t="n"/>
-      <c r="AR28" s="35" t="n"/>
-      <c r="AS28" s="36" t="n"/>
-      <c r="AT28" s="35" t="n"/>
-      <c r="AU28" s="35" t="n"/>
-    </row>
-    <row r="29" ht="24" customHeight="1" s="71">
-      <c r="A29" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sd45dbbc9fcb64ef4a78670e4fe959d40T.png")</f>
-        <v/>
-      </c>
-      <c r="D29" s="18" t="inlineStr">
-        <is>
-          <t>Windshield Sunshade Front Motorhome Thermal Windscreen Screen Cover Fo…</t>
-        </is>
-      </c>
-      <c r="E29" s="12" t="inlineStr">
-        <is>
-          <t>AliExpress: US $19.67. Vår räkning: landad ca 283 kr, tänkt butikspris 699 kr. Originaltitel: Windshield Sunshade Front Motorhome Thermal Windscreen Screen Cover For Fiat Ducato Peugeot Boxer Citroen Relay RV Cover</t>
-        </is>
-      </c>
-      <c r="H29" s="13" t="n"/>
-      <c r="I29" s="14" t="inlineStr">
-        <is>
-          <t>SWEDEN</t>
-        </is>
-      </c>
-      <c r="J29" s="15" t="n"/>
-      <c r="K29" s="15" t="n"/>
-      <c r="L29" s="16" t="n"/>
-      <c r="M29" s="14" t="n"/>
-      <c r="N29" s="17" t="inlineStr">
-        <is>
-          <t>https://www.aliexpress.com/item/1005011618553986.html</t>
-        </is>
-      </c>
-      <c r="Q29" s="18" t="n"/>
-      <c r="R29" s="19" t="n">
-        <v>100</v>
-      </c>
-      <c r="S29" s="15" t="n"/>
-      <c r="T29" s="15" t="n"/>
-      <c r="U29" s="16" t="n"/>
-      <c r="V29" s="48" t="n"/>
-      <c r="W29" s="48" t="n"/>
-      <c r="X29" s="21" t="n"/>
-      <c r="Y29" s="15" t="n"/>
-      <c r="Z29" s="15" t="n"/>
-      <c r="AA29" s="16" t="n"/>
-      <c r="AB29" s="48" t="n"/>
-      <c r="AC29" s="48" t="n"/>
-      <c r="AD29" s="22" t="n"/>
-      <c r="AE29" s="15" t="n"/>
-      <c r="AF29" s="15" t="n"/>
-      <c r="AG29" s="16" t="n"/>
-      <c r="AH29" s="48" t="n"/>
-      <c r="AI29" s="48" t="n"/>
-      <c r="AJ29" s="23" t="n"/>
-      <c r="AK29" s="15" t="n"/>
-      <c r="AL29" s="15" t="n"/>
-      <c r="AM29" s="16" t="n"/>
-      <c r="AN29" s="25" t="n"/>
-      <c r="AO29" s="48" t="n"/>
-      <c r="AP29" s="23" t="n"/>
-      <c r="AQ29" s="15" t="n"/>
-      <c r="AR29" s="15" t="n"/>
-      <c r="AS29" s="16" t="n"/>
-      <c r="AT29" s="25" t="n"/>
-      <c r="AU29" s="26" t="n"/>
-    </row>
-    <row r="30" ht="25.5" customHeight="1" s="71">
-      <c r="D30" s="18" t="n"/>
-      <c r="J30" s="15" t="n"/>
-      <c r="K30" s="15" t="n"/>
-      <c r="L30" s="16" t="n"/>
-      <c r="R30" s="19" t="n">
-        <v>200</v>
-      </c>
-      <c r="S30" s="15" t="n"/>
-      <c r="T30" s="15" t="n"/>
-      <c r="U30" s="16" t="n"/>
-      <c r="X30" s="21" t="n"/>
-      <c r="Y30" s="15" t="n"/>
-      <c r="Z30" s="15" t="n"/>
-      <c r="AA30" s="16" t="n"/>
-      <c r="AD30" s="22" t="n"/>
-      <c r="AE30" s="15" t="n"/>
-      <c r="AF30" s="15" t="n"/>
-      <c r="AG30" s="16" t="n"/>
-      <c r="AH30" s="48" t="n"/>
-      <c r="AI30" s="48" t="n"/>
-      <c r="AJ30" s="23" t="n"/>
-      <c r="AK30" s="15" t="n"/>
-      <c r="AL30" s="15" t="n"/>
-      <c r="AM30" s="16" t="n"/>
-      <c r="AP30" s="23" t="n"/>
-      <c r="AQ30" s="15" t="n"/>
-      <c r="AR30" s="15" t="n"/>
-      <c r="AS30" s="16" t="n"/>
-    </row>
-    <row r="31" s="71">
-      <c r="D31" s="18" t="n"/>
-      <c r="J31" s="15" t="n"/>
-      <c r="K31" s="15" t="n"/>
-      <c r="L31" s="16" t="n"/>
-      <c r="R31" s="19" t="n">
-        <v>300</v>
-      </c>
-      <c r="S31" s="15" t="n"/>
-      <c r="T31" s="15" t="n"/>
-      <c r="U31" s="16" t="n"/>
-      <c r="X31" s="21" t="n"/>
-      <c r="Y31" s="15" t="n"/>
-      <c r="Z31" s="15" t="n"/>
-      <c r="AA31" s="16" t="n"/>
-      <c r="AD31" s="22" t="n"/>
-      <c r="AE31" s="15" t="n"/>
-      <c r="AF31" s="15" t="n"/>
-      <c r="AG31" s="16" t="n"/>
-      <c r="AH31" s="48" t="n"/>
-      <c r="AI31" s="48" t="n"/>
-      <c r="AJ31" s="23" t="n"/>
-      <c r="AK31" s="15" t="n"/>
-      <c r="AL31" s="15" t="n"/>
-      <c r="AM31" s="16" t="n"/>
-      <c r="AP31" s="23" t="n"/>
-      <c r="AQ31" s="15" t="n"/>
-      <c r="AR31" s="15" t="n"/>
-      <c r="AS31" s="16" t="n"/>
-    </row>
-    <row r="32" ht="6.75" customHeight="1" s="71">
-      <c r="A32" s="27" t="n"/>
-      <c r="B32" s="27" t="n"/>
-      <c r="C32" s="27" t="n"/>
-      <c r="D32" s="27" t="n"/>
-      <c r="E32" s="27" t="n"/>
-      <c r="F32" s="27" t="n"/>
-      <c r="G32" s="27" t="n"/>
-      <c r="H32" s="35" t="n"/>
-      <c r="I32" s="35" t="n"/>
-      <c r="J32" s="36" t="n"/>
-      <c r="K32" s="36" t="n"/>
-      <c r="L32" s="36" t="n"/>
-      <c r="M32" s="35" t="n"/>
-      <c r="N32" s="30" t="n"/>
-      <c r="O32" s="30" t="n"/>
-      <c r="P32" s="30" t="n"/>
-      <c r="Q32" s="30" t="n"/>
-      <c r="R32" s="35" t="n"/>
-      <c r="S32" s="35" t="n"/>
-      <c r="T32" s="35" t="n"/>
-      <c r="U32" s="35" t="n"/>
-      <c r="V32" s="35" t="n"/>
-      <c r="W32" s="35" t="n"/>
-      <c r="X32" s="31" t="n"/>
-      <c r="Y32" s="35" t="n"/>
-      <c r="Z32" s="35" t="n"/>
-      <c r="AA32" s="36" t="n"/>
-      <c r="AB32" s="35" t="n"/>
-      <c r="AC32" s="35" t="n"/>
-      <c r="AD32" s="32" t="n"/>
-      <c r="AE32" s="35" t="n"/>
-      <c r="AF32" s="35" t="n"/>
-      <c r="AG32" s="36" t="n"/>
-      <c r="AH32" s="35" t="n"/>
-      <c r="AI32" s="35" t="n"/>
-      <c r="AJ32" s="34" t="n"/>
-      <c r="AK32" s="35" t="n"/>
-      <c r="AL32" s="35" t="n"/>
-      <c r="AM32" s="36" t="n"/>
-      <c r="AN32" s="35" t="n"/>
-      <c r="AO32" s="35" t="n"/>
-      <c r="AP32" s="34" t="n"/>
-      <c r="AQ32" s="35" t="n"/>
-      <c r="AR32" s="35" t="n"/>
-      <c r="AS32" s="36" t="n"/>
-      <c r="AT32" s="35" t="n"/>
-      <c r="AU32" s="35" t="n"/>
-    </row>
-    <row r="33" ht="24" customHeight="1" s="71">
-      <c r="A33" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sc87ec94ba4b94ae1b0f39ca26cfcad8dT.png")</f>
-        <v/>
-      </c>
-      <c r="D33" s="18" t="inlineStr">
-        <is>
-          <t>Solar Alarm IP65 Waterproof PIR Motion Detection Alarm with Siren and …</t>
-        </is>
-      </c>
-      <c r="E33" s="12" t="inlineStr">
-        <is>
-          <t>AliExpress: US $23.07. Vår räkning: landad ca 332 kr, tänkt butikspris 799 kr. Originaltitel: Solar Alarm IP65 Waterproof PIR Motion Detection Alarm with Siren and Strobe Light For Home Security Alarm System</t>
-        </is>
-      </c>
-      <c r="H33" s="13" t="n"/>
-      <c r="I33" s="14" t="inlineStr">
-        <is>
-          <t>SWEDEN</t>
-        </is>
-      </c>
-      <c r="J33" s="15" t="n"/>
-      <c r="K33" s="15" t="n"/>
-      <c r="L33" s="16" t="n"/>
-      <c r="M33" s="14" t="n"/>
-      <c r="N33" s="17" t="inlineStr">
-        <is>
-          <t>https://www.aliexpress.com/item/1005012241693262.html</t>
-        </is>
-      </c>
-      <c r="Q33" s="18" t="n"/>
-      <c r="R33" s="19" t="n">
-        <v>100</v>
-      </c>
-      <c r="S33" s="15" t="n"/>
-      <c r="T33" s="15" t="n"/>
-      <c r="U33" s="16" t="n"/>
-      <c r="V33" s="48" t="n"/>
-      <c r="W33" s="48" t="n"/>
-      <c r="X33" s="21" t="n"/>
-      <c r="Y33" s="15" t="n"/>
-      <c r="Z33" s="15" t="n"/>
-      <c r="AA33" s="16" t="n"/>
-      <c r="AB33" s="48" t="n"/>
-      <c r="AC33" s="48" t="n"/>
-      <c r="AD33" s="22" t="n"/>
-      <c r="AE33" s="15" t="n"/>
-      <c r="AF33" s="15" t="n"/>
-      <c r="AG33" s="16" t="n"/>
-      <c r="AH33" s="48" t="n"/>
-      <c r="AI33" s="48" t="n"/>
-      <c r="AJ33" s="23" t="n"/>
-      <c r="AK33" s="15" t="n"/>
-      <c r="AL33" s="15" t="n"/>
-      <c r="AM33" s="16" t="n"/>
-      <c r="AN33" s="25" t="n"/>
-      <c r="AO33" s="48" t="n"/>
-      <c r="AP33" s="23" t="n"/>
-      <c r="AQ33" s="15" t="n"/>
-      <c r="AR33" s="15" t="n"/>
-      <c r="AS33" s="16" t="n"/>
-      <c r="AT33" s="25" t="n"/>
-      <c r="AU33" s="26" t="n"/>
-    </row>
-    <row r="34" ht="25.5" customHeight="1" s="71">
-      <c r="D34" s="18" t="n"/>
-      <c r="J34" s="15" t="n"/>
-      <c r="K34" s="15" t="n"/>
-      <c r="L34" s="16" t="n"/>
-      <c r="R34" s="19" t="n">
-        <v>200</v>
-      </c>
-      <c r="S34" s="15" t="n"/>
-      <c r="T34" s="15" t="n"/>
-      <c r="U34" s="16" t="n"/>
-      <c r="X34" s="21" t="n"/>
-      <c r="Y34" s="15" t="n"/>
-      <c r="Z34" s="15" t="n"/>
-      <c r="AA34" s="16" t="n"/>
-      <c r="AD34" s="22" t="n"/>
-      <c r="AE34" s="15" t="n"/>
-      <c r="AF34" s="15" t="n"/>
-      <c r="AG34" s="16" t="n"/>
-      <c r="AH34" s="48" t="n"/>
-      <c r="AI34" s="48" t="n"/>
-      <c r="AJ34" s="23" t="n"/>
-      <c r="AK34" s="15" t="n"/>
-      <c r="AL34" s="15" t="n"/>
-      <c r="AM34" s="16" t="n"/>
-      <c r="AP34" s="23" t="n"/>
-      <c r="AQ34" s="15" t="n"/>
-      <c r="AR34" s="15" t="n"/>
-      <c r="AS34" s="16" t="n"/>
-    </row>
-    <row r="35" s="71">
-      <c r="D35" s="18" t="n"/>
-      <c r="J35" s="15" t="n"/>
-      <c r="K35" s="15" t="n"/>
-      <c r="L35" s="16" t="n"/>
-      <c r="R35" s="19" t="n">
-        <v>300</v>
-      </c>
-      <c r="S35" s="15" t="n"/>
-      <c r="T35" s="15" t="n"/>
-      <c r="U35" s="16" t="n"/>
-      <c r="X35" s="21" t="n"/>
-      <c r="Y35" s="15" t="n"/>
-      <c r="Z35" s="15" t="n"/>
-      <c r="AA35" s="16" t="n"/>
-      <c r="AD35" s="22" t="n"/>
-      <c r="AE35" s="15" t="n"/>
-      <c r="AF35" s="15" t="n"/>
-      <c r="AG35" s="16" t="n"/>
-      <c r="AH35" s="48" t="n"/>
-      <c r="AI35" s="48" t="n"/>
-      <c r="AJ35" s="23" t="n"/>
-      <c r="AK35" s="15" t="n"/>
-      <c r="AL35" s="15" t="n"/>
-      <c r="AM35" s="16" t="n"/>
-      <c r="AP35" s="23" t="n"/>
-      <c r="AQ35" s="15" t="n"/>
-      <c r="AR35" s="15" t="n"/>
-      <c r="AS35" s="16" t="n"/>
-    </row>
-    <row r="36" ht="6.75" customHeight="1" s="71">
-      <c r="A36" s="27" t="n"/>
-      <c r="B36" s="27" t="n"/>
-      <c r="C36" s="27" t="n"/>
-      <c r="D36" s="27" t="n"/>
-      <c r="E36" s="27" t="n"/>
-      <c r="F36" s="27" t="n"/>
-      <c r="G36" s="27" t="n"/>
-      <c r="H36" s="35" t="n"/>
-      <c r="I36" s="35" t="n"/>
-      <c r="J36" s="36" t="n"/>
-      <c r="K36" s="36" t="n"/>
-      <c r="L36" s="36" t="n"/>
-      <c r="M36" s="35" t="n"/>
-      <c r="N36" s="30" t="n"/>
-      <c r="O36" s="30" t="n"/>
-      <c r="P36" s="30" t="n"/>
-      <c r="Q36" s="30" t="n"/>
-      <c r="R36" s="35" t="n"/>
-      <c r="S36" s="35" t="n"/>
-      <c r="T36" s="35" t="n"/>
-      <c r="U36" s="35" t="n"/>
-      <c r="V36" s="35" t="n"/>
-      <c r="W36" s="35" t="n"/>
-      <c r="X36" s="31" t="n"/>
-      <c r="Y36" s="35" t="n"/>
-      <c r="Z36" s="35" t="n"/>
-      <c r="AA36" s="36" t="n"/>
-      <c r="AB36" s="35" t="n"/>
-      <c r="AC36" s="35" t="n"/>
-      <c r="AD36" s="32" t="n"/>
-      <c r="AE36" s="35" t="n"/>
-      <c r="AF36" s="35" t="n"/>
-      <c r="AG36" s="36" t="n"/>
-      <c r="AH36" s="35" t="n"/>
-      <c r="AI36" s="35" t="n"/>
-      <c r="AJ36" s="34" t="n"/>
-      <c r="AK36" s="35" t="n"/>
-      <c r="AL36" s="35" t="n"/>
-      <c r="AM36" s="36" t="n"/>
-      <c r="AN36" s="35" t="n"/>
-      <c r="AO36" s="35" t="n"/>
-      <c r="AP36" s="34" t="n"/>
-      <c r="AQ36" s="35" t="n"/>
-      <c r="AR36" s="35" t="n"/>
-      <c r="AS36" s="36" t="n"/>
-      <c r="AT36" s="35" t="n"/>
-      <c r="AU36" s="35" t="n"/>
-    </row>
+    <row r="25" ht="22.5" customHeight="1" s="71"/>
+    <row r="26" ht="22.5" customHeight="1" s="71"/>
+    <row r="27" ht="22.5" customHeight="1" s="71"/>
+    <row r="28" ht="6.75" customHeight="1" s="71"/>
+    <row r="29" ht="15.75" customHeight="1" s="71"/>
+    <row r="30" ht="15.75" customHeight="1" s="71"/>
+    <row r="31" ht="15.75" customHeight="1" s="71"/>
+    <row r="32" ht="15.75" customHeight="1" s="71"/>
+    <row r="33" ht="15.75" customHeight="1" s="71"/>
+    <row r="34" ht="15.75" customHeight="1" s="71"/>
+    <row r="35" ht="15.75" customHeight="1" s="71"/>
+    <row r="36" ht="15.75" customHeight="1" s="71"/>
     <row r="37" ht="15.75" customHeight="1" s="71"/>
     <row r="38" ht="15.75" customHeight="1" s="71"/>
     <row r="39" ht="15.75" customHeight="1" s="71"/>
@@ -3374,7 +2867,7 @@
     <row r="999" ht="15.75" customHeight="1" s="71"/>
     <row r="1000" ht="15.75" customHeight="1" s="71"/>
   </sheetData>
-  <mergeCells count="73">
+  <mergeCells count="52">
     <mergeCell ref="I5:I7"/>
     <mergeCell ref="E5:G7"/>
     <mergeCell ref="Q9:Q11"/>
@@ -3384,70 +2877,49 @@
     <mergeCell ref="L3:L4"/>
     <mergeCell ref="E13:G15"/>
     <mergeCell ref="X3:AC3"/>
-    <mergeCell ref="M33:M35"/>
     <mergeCell ref="N21:P23"/>
-    <mergeCell ref="I29:I31"/>
     <mergeCell ref="N5:P7"/>
     <mergeCell ref="H13:H15"/>
     <mergeCell ref="E3:G4"/>
-    <mergeCell ref="A25:C27"/>
     <mergeCell ref="AJ3:AO3"/>
-    <mergeCell ref="N33:P35"/>
     <mergeCell ref="M17:M19"/>
     <mergeCell ref="I13:I15"/>
     <mergeCell ref="Q17:Q19"/>
     <mergeCell ref="E9:G11"/>
     <mergeCell ref="R3:W3"/>
     <mergeCell ref="A21:C23"/>
-    <mergeCell ref="M29:M31"/>
     <mergeCell ref="A1:AO1"/>
     <mergeCell ref="M3:M4"/>
     <mergeCell ref="I3:I4"/>
     <mergeCell ref="Q13:Q15"/>
     <mergeCell ref="N13:P15"/>
     <mergeCell ref="N17:P19"/>
-    <mergeCell ref="Q25:Q27"/>
     <mergeCell ref="A17:C19"/>
-    <mergeCell ref="H33:H35"/>
     <mergeCell ref="H5:H7"/>
-    <mergeCell ref="N29:P31"/>
     <mergeCell ref="I9:I11"/>
-    <mergeCell ref="A33:C35"/>
-    <mergeCell ref="A29:C31"/>
     <mergeCell ref="A5:C7"/>
     <mergeCell ref="N3:P4"/>
     <mergeCell ref="M9:M11"/>
     <mergeCell ref="M5:M7"/>
-    <mergeCell ref="H29:H31"/>
     <mergeCell ref="A13:C15"/>
     <mergeCell ref="Q21:Q23"/>
-    <mergeCell ref="H25:H27"/>
     <mergeCell ref="H3:H4"/>
     <mergeCell ref="N9:P11"/>
     <mergeCell ref="J3:J4"/>
-    <mergeCell ref="Q33:Q35"/>
     <mergeCell ref="A3:C4"/>
     <mergeCell ref="AD3:AI3"/>
-    <mergeCell ref="E25:G27"/>
     <mergeCell ref="E21:G23"/>
     <mergeCell ref="Q5:Q7"/>
     <mergeCell ref="AP3:AU3"/>
     <mergeCell ref="H9:H11"/>
     <mergeCell ref="A2:AO2"/>
-    <mergeCell ref="E33:G35"/>
     <mergeCell ref="K3:K4"/>
     <mergeCell ref="A9:C11"/>
     <mergeCell ref="H21:H23"/>
-    <mergeCell ref="I25:I27"/>
-    <mergeCell ref="M25:M27"/>
     <mergeCell ref="Q3:Q4"/>
-    <mergeCell ref="Q29:Q31"/>
     <mergeCell ref="I21:I23"/>
     <mergeCell ref="E17:G19"/>
-    <mergeCell ref="N25:P27"/>
-    <mergeCell ref="I33:I35"/>
     <mergeCell ref="M13:M15"/>
-    <mergeCell ref="E29:G31"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId1"/>

</xml_diff>

<commit_message>
produktjakt: karantan pa sokord sa samma hylla inte kors om
Axel behöll sotsetet och batkapellstottan och kande igen resten. Rotorsaken ar
sokorden: samma ord ger samma hylla, och da kommer samma vara tillbaka fran en
ny saljare med nytt product_id — sedda.json ser det aldrig.

hitta.py har nu KARANTAN_DAGAR = 14. Anvanda sokord loggas i anvanda-sokord.json
och plockas bort ur poolen tills karantanen gatt ut; ar alla ord forbrukade
slapps sparren hellre an att leverera tomt. Dagens 28 ord ar inlagda.

Dagens leverans: 2 produkter, de Axel valde.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016jBJVGuyny8S3j2XPSM26Z
</commit_message>
<xml_diff>
--- a/produktjakt/korningar/2026-09-09/Leverantorsoffert-2026-09-09.xlsx
+++ b/produktjakt/korningar/2026-09-09/Leverantorsoffert-2026-09-09.xlsx
@@ -732,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU24"/>
+  <dimension ref="A1:AU12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="18" customWidth="1" style="71" min="1" max="1"/>
@@ -767,7 +767,7 @@
   <sheetData>
     <row r="1" ht="27.75" customHeight="1" s="71">
       <c r="A1" s="1" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AP1" s="1" t="n"/>
       <c r="AQ1" s="1" t="n"/>
@@ -1200,17 +1200,17 @@
     </row>
     <row r="9" ht="24" customHeight="1" s="71">
       <c r="A9" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S20416daaf99f4237ab753083a39afac5H.jpg")</f>
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sf82b0d4f34464eaca317489c4e31f25f8.jpg")</f>
         <v/>
       </c>
       <c r="D9" s="18" t="inlineStr">
         <is>
-          <t>Winter Warm Waterproof Stray Cat Dog House Foldable Washable Pet Cave …</t>
+          <t>Professional Telescopic Boat Cover Support Pole Windproof Adjustable H…</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $21.66. Vår räkning: landad ca 312 kr, tänkt butikspris 799 kr. Originaltitel: Winter Warm Waterproof Stray Cat Dog House Foldable Washable Pet Cave Outdoor Shelter Sleeping Bed for Small Puppy Pet Supplies</t>
+          <t>AliExpress: US $10.77. Vår räkning: landad ca 155 kr, tänkt butikspris 399 kr. Originaltitel: Professional Telescopic Boat Cover Support Pole Windproof Adjustable Height 22"-70" Heavy-Duty Steel/Aluminum for Pontoon Patio</t>
         </is>
       </c>
       <c r="H9" s="13" t="n"/>
@@ -1225,7 +1225,7 @@
       <c r="M9" s="14" t="n"/>
       <c r="N9" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005012414077421.html</t>
+          <t>https://www.aliexpress.com/item/1005009100129778.html</t>
         </is>
       </c>
       <c r="Q9" s="18" t="n"/>
@@ -1371,525 +1371,18 @@
       <c r="AT12" s="35" t="n"/>
       <c r="AU12" s="35" t="n"/>
     </row>
-    <row r="13" ht="24" customHeight="1" s="71">
-      <c r="A13" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sf82b0d4f34464eaca317489c4e31f25f8.jpg")</f>
-        <v/>
-      </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>Professional Telescopic Boat Cover Support Pole Windproof Adjustable H…</t>
-        </is>
-      </c>
-      <c r="E13" s="12" t="inlineStr">
-        <is>
-          <t>AliExpress: US $10.77. Vår räkning: landad ca 155 kr, tänkt butikspris 399 kr. Originaltitel: Professional Telescopic Boat Cover Support Pole Windproof Adjustable Height 22"-70" Heavy-Duty Steel/Aluminum for Pontoon Patio</t>
-        </is>
-      </c>
-      <c r="H13" s="13" t="n"/>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>SWEDEN</t>
-        </is>
-      </c>
-      <c r="J13" s="15" t="n"/>
-      <c r="K13" s="15" t="n"/>
-      <c r="L13" s="16" t="n"/>
-      <c r="M13" s="14" t="n"/>
-      <c r="N13" s="17" t="inlineStr">
-        <is>
-          <t>https://www.aliexpress.com/item/1005009100129778.html</t>
-        </is>
-      </c>
-      <c r="Q13" s="18" t="n"/>
-      <c r="R13" s="19" t="n">
-        <v>100</v>
-      </c>
-      <c r="S13" s="15" t="n"/>
-      <c r="T13" s="15" t="n"/>
-      <c r="U13" s="16" t="n"/>
-      <c r="V13" s="48" t="n"/>
-      <c r="W13" s="48" t="n"/>
-      <c r="X13" s="21" t="n"/>
-      <c r="Y13" s="15" t="n"/>
-      <c r="Z13" s="15" t="n"/>
-      <c r="AA13" s="16" t="n"/>
-      <c r="AB13" s="48" t="n"/>
-      <c r="AC13" s="48" t="n"/>
-      <c r="AD13" s="22" t="n"/>
-      <c r="AE13" s="15" t="n"/>
-      <c r="AF13" s="15" t="n"/>
-      <c r="AG13" s="16" t="n"/>
-      <c r="AH13" s="48" t="n"/>
-      <c r="AI13" s="48" t="n"/>
-      <c r="AJ13" s="23" t="n"/>
-      <c r="AK13" s="15" t="n"/>
-      <c r="AL13" s="15" t="n"/>
-      <c r="AM13" s="16" t="n"/>
-      <c r="AN13" s="25" t="n"/>
-      <c r="AO13" s="48" t="n"/>
-      <c r="AP13" s="23" t="n"/>
-      <c r="AQ13" s="15" t="n"/>
-      <c r="AR13" s="15" t="n"/>
-      <c r="AS13" s="16" t="n"/>
-      <c r="AT13" s="25" t="n"/>
-      <c r="AU13" s="26" t="n"/>
-    </row>
-    <row r="14" ht="25.5" customHeight="1" s="71">
-      <c r="D14" s="18" t="n"/>
-      <c r="J14" s="15" t="n"/>
-      <c r="K14" s="15" t="n"/>
-      <c r="L14" s="16" t="n"/>
-      <c r="R14" s="19" t="n">
-        <v>200</v>
-      </c>
-      <c r="S14" s="15" t="n"/>
-      <c r="T14" s="15" t="n"/>
-      <c r="U14" s="16" t="n"/>
-      <c r="X14" s="21" t="n"/>
-      <c r="Y14" s="15" t="n"/>
-      <c r="Z14" s="15" t="n"/>
-      <c r="AA14" s="16" t="n"/>
-      <c r="AD14" s="22" t="n"/>
-      <c r="AE14" s="15" t="n"/>
-      <c r="AF14" s="15" t="n"/>
-      <c r="AG14" s="16" t="n"/>
-      <c r="AH14" s="48" t="n"/>
-      <c r="AI14" s="48" t="n"/>
-      <c r="AJ14" s="23" t="n"/>
-      <c r="AK14" s="15" t="n"/>
-      <c r="AL14" s="15" t="n"/>
-      <c r="AM14" s="16" t="n"/>
-      <c r="AP14" s="23" t="n"/>
-      <c r="AQ14" s="15" t="n"/>
-      <c r="AR14" s="15" t="n"/>
-      <c r="AS14" s="16" t="n"/>
-    </row>
-    <row r="15" s="71">
-      <c r="D15" s="18" t="n"/>
-      <c r="J15" s="15" t="n"/>
-      <c r="K15" s="15" t="n"/>
-      <c r="L15" s="16" t="n"/>
-      <c r="R15" s="19" t="n">
-        <v>300</v>
-      </c>
-      <c r="S15" s="15" t="n"/>
-      <c r="T15" s="15" t="n"/>
-      <c r="U15" s="16" t="n"/>
-      <c r="X15" s="21" t="n"/>
-      <c r="Y15" s="15" t="n"/>
-      <c r="Z15" s="15" t="n"/>
-      <c r="AA15" s="16" t="n"/>
-      <c r="AD15" s="22" t="n"/>
-      <c r="AE15" s="15" t="n"/>
-      <c r="AF15" s="15" t="n"/>
-      <c r="AG15" s="16" t="n"/>
-      <c r="AH15" s="48" t="n"/>
-      <c r="AI15" s="48" t="n"/>
-      <c r="AJ15" s="23" t="n"/>
-      <c r="AK15" s="15" t="n"/>
-      <c r="AL15" s="15" t="n"/>
-      <c r="AM15" s="16" t="n"/>
-      <c r="AP15" s="23" t="n"/>
-      <c r="AQ15" s="15" t="n"/>
-      <c r="AR15" s="15" t="n"/>
-      <c r="AS15" s="16" t="n"/>
-    </row>
-    <row r="16" ht="6.75" customHeight="1" s="71">
-      <c r="A16" s="27" t="n"/>
-      <c r="B16" s="27" t="n"/>
-      <c r="C16" s="27" t="n"/>
-      <c r="D16" s="27" t="n"/>
-      <c r="E16" s="27" t="n"/>
-      <c r="F16" s="27" t="n"/>
-      <c r="G16" s="27" t="n"/>
-      <c r="H16" s="35" t="n"/>
-      <c r="I16" s="35" t="n"/>
-      <c r="J16" s="36" t="n"/>
-      <c r="K16" s="36" t="n"/>
-      <c r="L16" s="36" t="n"/>
-      <c r="M16" s="35" t="n"/>
-      <c r="N16" s="30" t="n"/>
-      <c r="O16" s="30" t="n"/>
-      <c r="P16" s="30" t="n"/>
-      <c r="Q16" s="30" t="n"/>
-      <c r="R16" s="35" t="n"/>
-      <c r="S16" s="35" t="n"/>
-      <c r="T16" s="35" t="n"/>
-      <c r="U16" s="35" t="n"/>
-      <c r="V16" s="35" t="n"/>
-      <c r="W16" s="35" t="n"/>
-      <c r="X16" s="31" t="n"/>
-      <c r="Y16" s="35" t="n"/>
-      <c r="Z16" s="35" t="n"/>
-      <c r="AA16" s="36" t="n"/>
-      <c r="AB16" s="35" t="n"/>
-      <c r="AC16" s="35" t="n"/>
-      <c r="AD16" s="32" t="n"/>
-      <c r="AE16" s="35" t="n"/>
-      <c r="AF16" s="35" t="n"/>
-      <c r="AG16" s="36" t="n"/>
-      <c r="AH16" s="35" t="n"/>
-      <c r="AI16" s="35" t="n"/>
-      <c r="AJ16" s="34" t="n"/>
-      <c r="AK16" s="35" t="n"/>
-      <c r="AL16" s="35" t="n"/>
-      <c r="AM16" s="36" t="n"/>
-      <c r="AN16" s="35" t="n"/>
-      <c r="AO16" s="35" t="n"/>
-      <c r="AP16" s="34" t="n"/>
-      <c r="AQ16" s="35" t="n"/>
-      <c r="AR16" s="35" t="n"/>
-      <c r="AS16" s="36" t="n"/>
-      <c r="AT16" s="35" t="n"/>
-      <c r="AU16" s="35" t="n"/>
-    </row>
-    <row r="17" ht="24" customHeight="1" s="71">
-      <c r="A17" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S1765e6b203364ba5b2b27145c16238989.jpg")</f>
-        <v/>
-      </c>
-      <c r="D17" s="18" t="inlineStr">
-        <is>
-          <t>Outboard Motor Flusher Muffs Kit with 16mm Quick Connect Fitting, Adju…</t>
-        </is>
-      </c>
-      <c r="E17" s="12" t="inlineStr">
-        <is>
-          <t>AliExpress: US $25.05. Vår räkning: landad ca 361 kr, tänkt butikspris 899 kr. Originaltitel: Outboard Motor Flusher Muffs Kit with 16mm Quick Connect Fitting, Adjustable Dual/Single Tube for Boat Motor Cleaning &amp; Test Run</t>
-        </is>
-      </c>
-      <c r="H17" s="13" t="n"/>
-      <c r="I17" s="14" t="inlineStr">
-        <is>
-          <t>SWEDEN</t>
-        </is>
-      </c>
-      <c r="J17" s="15" t="n"/>
-      <c r="K17" s="15" t="n"/>
-      <c r="L17" s="16" t="n"/>
-      <c r="M17" s="14" t="n"/>
-      <c r="N17" s="17" t="inlineStr">
-        <is>
-          <t>https://www.aliexpress.com/item/1005011764722846.html</t>
-        </is>
-      </c>
-      <c r="Q17" s="18" t="n"/>
-      <c r="R17" s="19" t="n">
-        <v>100</v>
-      </c>
-      <c r="S17" s="15" t="n"/>
-      <c r="T17" s="15" t="n"/>
-      <c r="U17" s="16" t="n"/>
-      <c r="V17" s="48" t="n"/>
-      <c r="W17" s="48" t="n"/>
-      <c r="X17" s="21" t="n"/>
-      <c r="Y17" s="15" t="n"/>
-      <c r="Z17" s="15" t="n"/>
-      <c r="AA17" s="16" t="n"/>
-      <c r="AB17" s="48" t="n"/>
-      <c r="AC17" s="48" t="n"/>
-      <c r="AD17" s="22" t="n"/>
-      <c r="AE17" s="15" t="n"/>
-      <c r="AF17" s="15" t="n"/>
-      <c r="AG17" s="16" t="n"/>
-      <c r="AH17" s="48" t="n"/>
-      <c r="AI17" s="48" t="n"/>
-      <c r="AJ17" s="23" t="n"/>
-      <c r="AK17" s="15" t="n"/>
-      <c r="AL17" s="15" t="n"/>
-      <c r="AM17" s="16" t="n"/>
-      <c r="AN17" s="25" t="n"/>
-      <c r="AO17" s="48" t="n"/>
-      <c r="AP17" s="23" t="n"/>
-      <c r="AQ17" s="15" t="n"/>
-      <c r="AR17" s="15" t="n"/>
-      <c r="AS17" s="16" t="n"/>
-      <c r="AT17" s="25" t="n"/>
-      <c r="AU17" s="26" t="n"/>
-    </row>
-    <row r="18" ht="25.5" customHeight="1" s="71">
-      <c r="D18" s="18" t="n"/>
-      <c r="J18" s="15" t="n"/>
-      <c r="K18" s="15" t="n"/>
-      <c r="L18" s="16" t="n"/>
-      <c r="R18" s="19" t="n">
-        <v>200</v>
-      </c>
-      <c r="S18" s="15" t="n"/>
-      <c r="T18" s="15" t="n"/>
-      <c r="U18" s="16" t="n"/>
-      <c r="X18" s="21" t="n"/>
-      <c r="Y18" s="15" t="n"/>
-      <c r="Z18" s="15" t="n"/>
-      <c r="AA18" s="16" t="n"/>
-      <c r="AD18" s="22" t="n"/>
-      <c r="AE18" s="15" t="n"/>
-      <c r="AF18" s="15" t="n"/>
-      <c r="AG18" s="16" t="n"/>
-      <c r="AH18" s="48" t="n"/>
-      <c r="AI18" s="48" t="n"/>
-      <c r="AJ18" s="23" t="n"/>
-      <c r="AK18" s="15" t="n"/>
-      <c r="AL18" s="15" t="n"/>
-      <c r="AM18" s="16" t="n"/>
-      <c r="AP18" s="23" t="n"/>
-      <c r="AQ18" s="15" t="n"/>
-      <c r="AR18" s="15" t="n"/>
-      <c r="AS18" s="16" t="n"/>
-    </row>
-    <row r="19" s="71">
-      <c r="D19" s="18" t="n"/>
-      <c r="J19" s="15" t="n"/>
-      <c r="K19" s="15" t="n"/>
-      <c r="L19" s="16" t="n"/>
-      <c r="R19" s="19" t="n">
-        <v>300</v>
-      </c>
-      <c r="S19" s="15" t="n"/>
-      <c r="T19" s="15" t="n"/>
-      <c r="U19" s="16" t="n"/>
-      <c r="X19" s="21" t="n"/>
-      <c r="Y19" s="15" t="n"/>
-      <c r="Z19" s="15" t="n"/>
-      <c r="AA19" s="16" t="n"/>
-      <c r="AD19" s="22" t="n"/>
-      <c r="AE19" s="15" t="n"/>
-      <c r="AF19" s="15" t="n"/>
-      <c r="AG19" s="16" t="n"/>
-      <c r="AH19" s="48" t="n"/>
-      <c r="AI19" s="48" t="n"/>
-      <c r="AJ19" s="23" t="n"/>
-      <c r="AK19" s="15" t="n"/>
-      <c r="AL19" s="15" t="n"/>
-      <c r="AM19" s="16" t="n"/>
-      <c r="AP19" s="23" t="n"/>
-      <c r="AQ19" s="15" t="n"/>
-      <c r="AR19" s="15" t="n"/>
-      <c r="AS19" s="16" t="n"/>
-    </row>
-    <row r="20" ht="6.75" customHeight="1" s="71">
-      <c r="A20" s="27" t="n"/>
-      <c r="B20" s="27" t="n"/>
-      <c r="C20" s="27" t="n"/>
-      <c r="D20" s="27" t="n"/>
-      <c r="E20" s="27" t="n"/>
-      <c r="F20" s="27" t="n"/>
-      <c r="G20" s="27" t="n"/>
-      <c r="H20" s="35" t="n"/>
-      <c r="I20" s="35" t="n"/>
-      <c r="J20" s="36" t="n"/>
-      <c r="K20" s="36" t="n"/>
-      <c r="L20" s="36" t="n"/>
-      <c r="M20" s="35" t="n"/>
-      <c r="N20" s="30" t="n"/>
-      <c r="O20" s="30" t="n"/>
-      <c r="P20" s="30" t="n"/>
-      <c r="Q20" s="30" t="n"/>
-      <c r="R20" s="35" t="n"/>
-      <c r="S20" s="35" t="n"/>
-      <c r="T20" s="35" t="n"/>
-      <c r="U20" s="35" t="n"/>
-      <c r="V20" s="35" t="n"/>
-      <c r="W20" s="35" t="n"/>
-      <c r="X20" s="31" t="n"/>
-      <c r="Y20" s="35" t="n"/>
-      <c r="Z20" s="35" t="n"/>
-      <c r="AA20" s="36" t="n"/>
-      <c r="AB20" s="35" t="n"/>
-      <c r="AC20" s="35" t="n"/>
-      <c r="AD20" s="32" t="n"/>
-      <c r="AE20" s="35" t="n"/>
-      <c r="AF20" s="35" t="n"/>
-      <c r="AG20" s="36" t="n"/>
-      <c r="AH20" s="35" t="n"/>
-      <c r="AI20" s="35" t="n"/>
-      <c r="AJ20" s="34" t="n"/>
-      <c r="AK20" s="35" t="n"/>
-      <c r="AL20" s="35" t="n"/>
-      <c r="AM20" s="36" t="n"/>
-      <c r="AN20" s="35" t="n"/>
-      <c r="AO20" s="35" t="n"/>
-      <c r="AP20" s="34" t="n"/>
-      <c r="AQ20" s="35" t="n"/>
-      <c r="AR20" s="35" t="n"/>
-      <c r="AS20" s="36" t="n"/>
-      <c r="AT20" s="35" t="n"/>
-      <c r="AU20" s="35" t="n"/>
-    </row>
-    <row r="21" ht="24" customHeight="1" s="71">
-      <c r="A21" s="10">
-        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sda69235967df40a5a5442b5e4f1323c5M.jpg")</f>
-        <v/>
-      </c>
-      <c r="D21" s="18" t="inlineStr">
-        <is>
-          <t>1/2 Pack Heavy Duty Steel Fence Post Repair Kit - Anchor Brackets &amp; Gr…</t>
-        </is>
-      </c>
-      <c r="E21" s="12" t="inlineStr">
-        <is>
-          <t>AliExpress: US $18.74. Vår räkning: landad ca 270 kr, tänkt butikspris 699 kr. Originaltitel: 1/2 Pack Heavy Duty Steel Fence Post Repair Kit - Anchor Brackets &amp; Ground Spike for Fixing Tilted/Broken Wooden Fence Posts</t>
-        </is>
-      </c>
-      <c r="H21" s="13" t="n"/>
-      <c r="I21" s="14" t="inlineStr">
-        <is>
-          <t>SWEDEN</t>
-        </is>
-      </c>
-      <c r="J21" s="15" t="n"/>
-      <c r="K21" s="15" t="n"/>
-      <c r="L21" s="16" t="n"/>
-      <c r="M21" s="14" t="n"/>
-      <c r="N21" s="17" t="inlineStr">
-        <is>
-          <t>https://www.aliexpress.com/item/1005009145737438.html</t>
-        </is>
-      </c>
-      <c r="Q21" s="18" t="n"/>
-      <c r="R21" s="19" t="n">
-        <v>100</v>
-      </c>
-      <c r="S21" s="15" t="n"/>
-      <c r="T21" s="15" t="n"/>
-      <c r="U21" s="16" t="n"/>
-      <c r="V21" s="48" t="n"/>
-      <c r="W21" s="48" t="n"/>
-      <c r="X21" s="21" t="n"/>
-      <c r="Y21" s="15" t="n"/>
-      <c r="Z21" s="15" t="n"/>
-      <c r="AA21" s="16" t="n"/>
-      <c r="AB21" s="48" t="n"/>
-      <c r="AC21" s="48" t="n"/>
-      <c r="AD21" s="22" t="n"/>
-      <c r="AE21" s="15" t="n"/>
-      <c r="AF21" s="15" t="n"/>
-      <c r="AG21" s="16" t="n"/>
-      <c r="AH21" s="48" t="n"/>
-      <c r="AI21" s="48" t="n"/>
-      <c r="AJ21" s="23" t="n"/>
-      <c r="AK21" s="15" t="n"/>
-      <c r="AL21" s="15" t="n"/>
-      <c r="AM21" s="16" t="n"/>
-      <c r="AN21" s="25" t="n"/>
-      <c r="AO21" s="48" t="n"/>
-      <c r="AP21" s="23" t="n"/>
-      <c r="AQ21" s="15" t="n"/>
-      <c r="AR21" s="15" t="n"/>
-      <c r="AS21" s="16" t="n"/>
-      <c r="AT21" s="25" t="n"/>
-      <c r="AU21" s="26" t="n"/>
-    </row>
-    <row r="22" ht="25.5" customHeight="1" s="71">
-      <c r="D22" s="18" t="n"/>
-      <c r="J22" s="15" t="n"/>
-      <c r="K22" s="15" t="n"/>
-      <c r="L22" s="16" t="n"/>
-      <c r="R22" s="19" t="n">
-        <v>200</v>
-      </c>
-      <c r="S22" s="15" t="n"/>
-      <c r="T22" s="15" t="n"/>
-      <c r="U22" s="16" t="n"/>
-      <c r="X22" s="21" t="n"/>
-      <c r="Y22" s="15" t="n"/>
-      <c r="Z22" s="15" t="n"/>
-      <c r="AA22" s="16" t="n"/>
-      <c r="AD22" s="22" t="n"/>
-      <c r="AE22" s="15" t="n"/>
-      <c r="AF22" s="15" t="n"/>
-      <c r="AG22" s="16" t="n"/>
-      <c r="AH22" s="48" t="n"/>
-      <c r="AI22" s="48" t="n"/>
-      <c r="AJ22" s="23" t="n"/>
-      <c r="AK22" s="15" t="n"/>
-      <c r="AL22" s="15" t="n"/>
-      <c r="AM22" s="16" t="n"/>
-      <c r="AP22" s="23" t="n"/>
-      <c r="AQ22" s="15" t="n"/>
-      <c r="AR22" s="15" t="n"/>
-      <c r="AS22" s="16" t="n"/>
-    </row>
-    <row r="23" s="71">
-      <c r="D23" s="18" t="n"/>
-      <c r="J23" s="15" t="n"/>
-      <c r="K23" s="15" t="n"/>
-      <c r="L23" s="16" t="n"/>
-      <c r="R23" s="19" t="n">
-        <v>300</v>
-      </c>
-      <c r="S23" s="15" t="n"/>
-      <c r="T23" s="15" t="n"/>
-      <c r="U23" s="16" t="n"/>
-      <c r="X23" s="21" t="n"/>
-      <c r="Y23" s="15" t="n"/>
-      <c r="Z23" s="15" t="n"/>
-      <c r="AA23" s="16" t="n"/>
-      <c r="AD23" s="22" t="n"/>
-      <c r="AE23" s="15" t="n"/>
-      <c r="AF23" s="15" t="n"/>
-      <c r="AG23" s="16" t="n"/>
-      <c r="AH23" s="48" t="n"/>
-      <c r="AI23" s="48" t="n"/>
-      <c r="AJ23" s="23" t="n"/>
-      <c r="AK23" s="15" t="n"/>
-      <c r="AL23" s="15" t="n"/>
-      <c r="AM23" s="16" t="n"/>
-      <c r="AP23" s="23" t="n"/>
-      <c r="AQ23" s="15" t="n"/>
-      <c r="AR23" s="15" t="n"/>
-      <c r="AS23" s="16" t="n"/>
-    </row>
-    <row r="24" ht="6.75" customHeight="1" s="71">
-      <c r="A24" s="27" t="n"/>
-      <c r="B24" s="27" t="n"/>
-      <c r="C24" s="27" t="n"/>
-      <c r="D24" s="27" t="n"/>
-      <c r="E24" s="27" t="n"/>
-      <c r="F24" s="27" t="n"/>
-      <c r="G24" s="27" t="n"/>
-      <c r="H24" s="35" t="n"/>
-      <c r="I24" s="35" t="n"/>
-      <c r="J24" s="36" t="n"/>
-      <c r="K24" s="36" t="n"/>
-      <c r="L24" s="36" t="n"/>
-      <c r="M24" s="35" t="n"/>
-      <c r="N24" s="30" t="n"/>
-      <c r="O24" s="30" t="n"/>
-      <c r="P24" s="30" t="n"/>
-      <c r="Q24" s="30" t="n"/>
-      <c r="R24" s="35" t="n"/>
-      <c r="S24" s="35" t="n"/>
-      <c r="T24" s="35" t="n"/>
-      <c r="U24" s="35" t="n"/>
-      <c r="V24" s="35" t="n"/>
-      <c r="W24" s="35" t="n"/>
-      <c r="X24" s="31" t="n"/>
-      <c r="Y24" s="35" t="n"/>
-      <c r="Z24" s="35" t="n"/>
-      <c r="AA24" s="36" t="n"/>
-      <c r="AB24" s="35" t="n"/>
-      <c r="AC24" s="35" t="n"/>
-      <c r="AD24" s="32" t="n"/>
-      <c r="AE24" s="35" t="n"/>
-      <c r="AF24" s="35" t="n"/>
-      <c r="AG24" s="36" t="n"/>
-      <c r="AH24" s="35" t="n"/>
-      <c r="AI24" s="35" t="n"/>
-      <c r="AJ24" s="34" t="n"/>
-      <c r="AK24" s="35" t="n"/>
-      <c r="AL24" s="35" t="n"/>
-      <c r="AM24" s="36" t="n"/>
-      <c r="AN24" s="35" t="n"/>
-      <c r="AO24" s="35" t="n"/>
-      <c r="AP24" s="34" t="n"/>
-      <c r="AQ24" s="35" t="n"/>
-      <c r="AR24" s="35" t="n"/>
-      <c r="AS24" s="36" t="n"/>
-      <c r="AT24" s="35" t="n"/>
-      <c r="AU24" s="35" t="n"/>
-    </row>
+    <row r="13" ht="22.5" customHeight="1" s="71"/>
+    <row r="14" ht="22.5" customHeight="1" s="71"/>
+    <row r="15" ht="22.5" customHeight="1" s="71"/>
+    <row r="16" ht="6.75" customHeight="1" s="71"/>
+    <row r="17" ht="22.5" customHeight="1" s="71"/>
+    <row r="18" ht="22.5" customHeight="1" s="71"/>
+    <row r="19" ht="22.5" customHeight="1" s="71"/>
+    <row r="20" ht="6.75" customHeight="1" s="71"/>
+    <row r="21" ht="22.5" customHeight="1" s="71"/>
+    <row r="22" ht="22.5" customHeight="1" s="71"/>
+    <row r="23" ht="22.5" customHeight="1" s="71"/>
+    <row r="24" ht="6.75" customHeight="1" s="71"/>
     <row r="25" ht="22.5" customHeight="1" s="71"/>
     <row r="26" ht="22.5" customHeight="1" s="71"/>
     <row r="27" ht="22.5" customHeight="1" s="71"/>
@@ -2867,63 +2360,39 @@
     <row r="999" ht="15.75" customHeight="1" s="71"/>
     <row r="1000" ht="15.75" customHeight="1" s="71"/>
   </sheetData>
-  <mergeCells count="52">
+  <mergeCells count="31">
     <mergeCell ref="I5:I7"/>
     <mergeCell ref="E5:G7"/>
     <mergeCell ref="Q9:Q11"/>
-    <mergeCell ref="H17:H19"/>
-    <mergeCell ref="I17:I19"/>
-    <mergeCell ref="M21:M23"/>
     <mergeCell ref="L3:L4"/>
-    <mergeCell ref="E13:G15"/>
     <mergeCell ref="X3:AC3"/>
-    <mergeCell ref="N21:P23"/>
     <mergeCell ref="N5:P7"/>
-    <mergeCell ref="H13:H15"/>
     <mergeCell ref="E3:G4"/>
     <mergeCell ref="AJ3:AO3"/>
-    <mergeCell ref="M17:M19"/>
-    <mergeCell ref="I13:I15"/>
-    <mergeCell ref="Q17:Q19"/>
     <mergeCell ref="E9:G11"/>
     <mergeCell ref="R3:W3"/>
-    <mergeCell ref="A21:C23"/>
     <mergeCell ref="A1:AO1"/>
     <mergeCell ref="M3:M4"/>
     <mergeCell ref="I3:I4"/>
-    <mergeCell ref="Q13:Q15"/>
-    <mergeCell ref="N13:P15"/>
-    <mergeCell ref="N17:P19"/>
-    <mergeCell ref="A17:C19"/>
     <mergeCell ref="H5:H7"/>
     <mergeCell ref="I9:I11"/>
     <mergeCell ref="A5:C7"/>
     <mergeCell ref="N3:P4"/>
     <mergeCell ref="M9:M11"/>
     <mergeCell ref="M5:M7"/>
-    <mergeCell ref="A13:C15"/>
-    <mergeCell ref="Q21:Q23"/>
     <mergeCell ref="H3:H4"/>
     <mergeCell ref="N9:P11"/>
     <mergeCell ref="J3:J4"/>
     <mergeCell ref="A3:C4"/>
     <mergeCell ref="AD3:AI3"/>
-    <mergeCell ref="E21:G23"/>
     <mergeCell ref="Q5:Q7"/>
     <mergeCell ref="AP3:AU3"/>
     <mergeCell ref="H9:H11"/>
     <mergeCell ref="A2:AO2"/>
     <mergeCell ref="K3:K4"/>
     <mergeCell ref="A9:C11"/>
-    <mergeCell ref="H21:H23"/>
     <mergeCell ref="Q3:Q4"/>
-    <mergeCell ref="I21:I23"/>
-    <mergeCell ref="E17:G19"/>
-    <mergeCell ref="M13:M15"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>

</xml_diff>

<commit_message>
produktjakt: grinden stryker inget fran offertarket
Axels beslut 2026-09-09: alla nio kandidater ska med pa arket, aven de sex som foll pa
wow-testet. Det ar ratt. Arket ar en forfragan, inte ett launchbeslut — att fraga
leverantoren om pris kostar ingenting, och leverantorens riktiga pris ar data vi annars
aldrig far. Flera av dagens domar hangde just pa prislaget, och det priset var var egen
rakning, inte leverantorens.

Grinden flyttar darfor ett steg: wow-testet avgor vad som LAUNCHAS, inte vad som
offereras. Domen skrivs i korningens STATUS.md sa att den som valjer ur offerten vet
vilka varor som saknar payoff i ett tystat flode.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016jBJVGuyny8S3j2XPSM26Z
</commit_message>
<xml_diff>
--- a/produktjakt/korningar/2026-09-09/Leverantorsoffert-2026-09-09.xlsx
+++ b/produktjakt/korningar/2026-09-09/Leverantorsoffert-2026-09-09.xlsx
@@ -732,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU16"/>
+  <dimension ref="A1:AU40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="18" customWidth="1" style="71" min="1" max="1"/>
@@ -767,7 +767,7 @@
   <sheetData>
     <row r="1" ht="27.75" customHeight="1" s="71">
       <c r="A1" s="1" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AP1" s="1" t="n"/>
       <c r="AQ1" s="1" t="n"/>
@@ -1544,30 +1544,1044 @@
       <c r="AT16" s="35" t="n"/>
       <c r="AU16" s="35" t="n"/>
     </row>
-    <row r="17" ht="22.5" customHeight="1" s="71"/>
-    <row r="18" ht="22.5" customHeight="1" s="71"/>
-    <row r="19" ht="22.5" customHeight="1" s="71"/>
-    <row r="20" ht="6.75" customHeight="1" s="71"/>
-    <row r="21" ht="22.5" customHeight="1" s="71"/>
-    <row r="22" ht="22.5" customHeight="1" s="71"/>
-    <row r="23" ht="22.5" customHeight="1" s="71"/>
-    <row r="24" ht="6.75" customHeight="1" s="71"/>
-    <row r="25" ht="22.5" customHeight="1" s="71"/>
-    <row r="26" ht="22.5" customHeight="1" s="71"/>
-    <row r="27" ht="22.5" customHeight="1" s="71"/>
-    <row r="28" ht="6.75" customHeight="1" s="71"/>
-    <row r="29" ht="15.75" customHeight="1" s="71"/>
-    <row r="30" ht="15.75" customHeight="1" s="71"/>
-    <row r="31" ht="15.75" customHeight="1" s="71"/>
-    <row r="32" ht="15.75" customHeight="1" s="71"/>
-    <row r="33" ht="15.75" customHeight="1" s="71"/>
-    <row r="34" ht="15.75" customHeight="1" s="71"/>
-    <row r="35" ht="15.75" customHeight="1" s="71"/>
-    <row r="36" ht="15.75" customHeight="1" s="71"/>
-    <row r="37" ht="15.75" customHeight="1" s="71"/>
-    <row r="38" ht="15.75" customHeight="1" s="71"/>
-    <row r="39" ht="15.75" customHeight="1" s="71"/>
-    <row r="40" ht="15.75" customHeight="1" s="71"/>
+    <row r="17" ht="24" customHeight="1" s="71">
+      <c r="A17" s="10">
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/Sb74de03bb0c04c87b52041a3cdae4e4eH.jpg")</f>
+        <v/>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>Gutter Cleaner MAX Use Of Any Hand Tool In The Scoop Coupler, Gutter C…</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>AliExpress: US $13.18. Vår räkning: landad ca 190 kr, tänkt butikspris 499 kr. Originaltitel: Gutter Cleaner MAX Use Of Any Hand Tool In The Scoop Coupler, Gutter Cleaning From The Ground, Roof And Ladders</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="n"/>
+      <c r="I17" s="14" t="inlineStr">
+        <is>
+          <t>SWEDEN</t>
+        </is>
+      </c>
+      <c r="J17" s="15" t="n"/>
+      <c r="K17" s="15" t="n"/>
+      <c r="L17" s="16" t="n"/>
+      <c r="M17" s="14" t="n"/>
+      <c r="N17" s="17" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.com/item/1005012694054863.html</t>
+        </is>
+      </c>
+      <c r="Q17" s="18" t="n"/>
+      <c r="R17" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="S17" s="15" t="n"/>
+      <c r="T17" s="15" t="n"/>
+      <c r="U17" s="16" t="n"/>
+      <c r="V17" s="48" t="n"/>
+      <c r="W17" s="48" t="n"/>
+      <c r="X17" s="21" t="n"/>
+      <c r="Y17" s="15" t="n"/>
+      <c r="Z17" s="15" t="n"/>
+      <c r="AA17" s="16" t="n"/>
+      <c r="AB17" s="48" t="n"/>
+      <c r="AC17" s="48" t="n"/>
+      <c r="AD17" s="22" t="n"/>
+      <c r="AE17" s="15" t="n"/>
+      <c r="AF17" s="15" t="n"/>
+      <c r="AG17" s="16" t="n"/>
+      <c r="AH17" s="48" t="n"/>
+      <c r="AI17" s="48" t="n"/>
+      <c r="AJ17" s="23" t="n"/>
+      <c r="AK17" s="15" t="n"/>
+      <c r="AL17" s="15" t="n"/>
+      <c r="AM17" s="16" t="n"/>
+      <c r="AN17" s="25" t="n"/>
+      <c r="AO17" s="48" t="n"/>
+      <c r="AP17" s="23" t="n"/>
+      <c r="AQ17" s="15" t="n"/>
+      <c r="AR17" s="15" t="n"/>
+      <c r="AS17" s="16" t="n"/>
+      <c r="AT17" s="25" t="n"/>
+      <c r="AU17" s="26" t="n"/>
+    </row>
+    <row r="18" ht="25.5" customHeight="1" s="71">
+      <c r="D18" s="18" t="n"/>
+      <c r="J18" s="15" t="n"/>
+      <c r="K18" s="15" t="n"/>
+      <c r="L18" s="16" t="n"/>
+      <c r="R18" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="S18" s="15" t="n"/>
+      <c r="T18" s="15" t="n"/>
+      <c r="U18" s="16" t="n"/>
+      <c r="X18" s="21" t="n"/>
+      <c r="Y18" s="15" t="n"/>
+      <c r="Z18" s="15" t="n"/>
+      <c r="AA18" s="16" t="n"/>
+      <c r="AD18" s="22" t="n"/>
+      <c r="AE18" s="15" t="n"/>
+      <c r="AF18" s="15" t="n"/>
+      <c r="AG18" s="16" t="n"/>
+      <c r="AH18" s="48" t="n"/>
+      <c r="AI18" s="48" t="n"/>
+      <c r="AJ18" s="23" t="n"/>
+      <c r="AK18" s="15" t="n"/>
+      <c r="AL18" s="15" t="n"/>
+      <c r="AM18" s="16" t="n"/>
+      <c r="AP18" s="23" t="n"/>
+      <c r="AQ18" s="15" t="n"/>
+      <c r="AR18" s="15" t="n"/>
+      <c r="AS18" s="16" t="n"/>
+    </row>
+    <row r="19" s="71">
+      <c r="D19" s="18" t="n"/>
+      <c r="J19" s="15" t="n"/>
+      <c r="K19" s="15" t="n"/>
+      <c r="L19" s="16" t="n"/>
+      <c r="R19" s="19" t="n">
+        <v>300</v>
+      </c>
+      <c r="S19" s="15" t="n"/>
+      <c r="T19" s="15" t="n"/>
+      <c r="U19" s="16" t="n"/>
+      <c r="X19" s="21" t="n"/>
+      <c r="Y19" s="15" t="n"/>
+      <c r="Z19" s="15" t="n"/>
+      <c r="AA19" s="16" t="n"/>
+      <c r="AD19" s="22" t="n"/>
+      <c r="AE19" s="15" t="n"/>
+      <c r="AF19" s="15" t="n"/>
+      <c r="AG19" s="16" t="n"/>
+      <c r="AH19" s="48" t="n"/>
+      <c r="AI19" s="48" t="n"/>
+      <c r="AJ19" s="23" t="n"/>
+      <c r="AK19" s="15" t="n"/>
+      <c r="AL19" s="15" t="n"/>
+      <c r="AM19" s="16" t="n"/>
+      <c r="AP19" s="23" t="n"/>
+      <c r="AQ19" s="15" t="n"/>
+      <c r="AR19" s="15" t="n"/>
+      <c r="AS19" s="16" t="n"/>
+    </row>
+    <row r="20" ht="6.75" customHeight="1" s="71">
+      <c r="A20" s="27" t="n"/>
+      <c r="B20" s="27" t="n"/>
+      <c r="C20" s="27" t="n"/>
+      <c r="D20" s="27" t="n"/>
+      <c r="E20" s="27" t="n"/>
+      <c r="F20" s="27" t="n"/>
+      <c r="G20" s="27" t="n"/>
+      <c r="H20" s="35" t="n"/>
+      <c r="I20" s="35" t="n"/>
+      <c r="J20" s="36" t="n"/>
+      <c r="K20" s="36" t="n"/>
+      <c r="L20" s="36" t="n"/>
+      <c r="M20" s="35" t="n"/>
+      <c r="N20" s="30" t="n"/>
+      <c r="O20" s="30" t="n"/>
+      <c r="P20" s="30" t="n"/>
+      <c r="Q20" s="30" t="n"/>
+      <c r="R20" s="35" t="n"/>
+      <c r="S20" s="35" t="n"/>
+      <c r="T20" s="35" t="n"/>
+      <c r="U20" s="35" t="n"/>
+      <c r="V20" s="35" t="n"/>
+      <c r="W20" s="35" t="n"/>
+      <c r="X20" s="31" t="n"/>
+      <c r="Y20" s="35" t="n"/>
+      <c r="Z20" s="35" t="n"/>
+      <c r="AA20" s="36" t="n"/>
+      <c r="AB20" s="35" t="n"/>
+      <c r="AC20" s="35" t="n"/>
+      <c r="AD20" s="32" t="n"/>
+      <c r="AE20" s="35" t="n"/>
+      <c r="AF20" s="35" t="n"/>
+      <c r="AG20" s="36" t="n"/>
+      <c r="AH20" s="35" t="n"/>
+      <c r="AI20" s="35" t="n"/>
+      <c r="AJ20" s="34" t="n"/>
+      <c r="AK20" s="35" t="n"/>
+      <c r="AL20" s="35" t="n"/>
+      <c r="AM20" s="36" t="n"/>
+      <c r="AN20" s="35" t="n"/>
+      <c r="AO20" s="35" t="n"/>
+      <c r="AP20" s="34" t="n"/>
+      <c r="AQ20" s="35" t="n"/>
+      <c r="AR20" s="35" t="n"/>
+      <c r="AS20" s="36" t="n"/>
+      <c r="AT20" s="35" t="n"/>
+      <c r="AU20" s="35" t="n"/>
+    </row>
+    <row r="21" ht="24" customHeight="1" s="71">
+      <c r="A21" s="10">
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S42dc5c6554c844a3ae5ff63df1f81a04E.jpg")</f>
+        <v/>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>For Standard Quart Bottles Lower Unit Gear Oil Pump Includes Metal Swi…</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>AliExpress: US $10.46. Vår räkning: landad ca 151 kr, tänkt butikspris 399 kr. Originaltitel: For Standard Quart Bottles Lower Unit Gear Oil Pump Includes Metal Swivel 8mm 10mm Adapters Fit Most Marine Boat Outboard Motors</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="n"/>
+      <c r="I21" s="14" t="inlineStr">
+        <is>
+          <t>SWEDEN</t>
+        </is>
+      </c>
+      <c r="J21" s="15" t="n"/>
+      <c r="K21" s="15" t="n"/>
+      <c r="L21" s="16" t="n"/>
+      <c r="M21" s="14" t="n"/>
+      <c r="N21" s="17" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.com/item/1005008249258612.html</t>
+        </is>
+      </c>
+      <c r="Q21" s="18" t="n"/>
+      <c r="R21" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="S21" s="15" t="n"/>
+      <c r="T21" s="15" t="n"/>
+      <c r="U21" s="16" t="n"/>
+      <c r="V21" s="48" t="n"/>
+      <c r="W21" s="48" t="n"/>
+      <c r="X21" s="21" t="n"/>
+      <c r="Y21" s="15" t="n"/>
+      <c r="Z21" s="15" t="n"/>
+      <c r="AA21" s="16" t="n"/>
+      <c r="AB21" s="48" t="n"/>
+      <c r="AC21" s="48" t="n"/>
+      <c r="AD21" s="22" t="n"/>
+      <c r="AE21" s="15" t="n"/>
+      <c r="AF21" s="15" t="n"/>
+      <c r="AG21" s="16" t="n"/>
+      <c r="AH21" s="48" t="n"/>
+      <c r="AI21" s="48" t="n"/>
+      <c r="AJ21" s="23" t="n"/>
+      <c r="AK21" s="15" t="n"/>
+      <c r="AL21" s="15" t="n"/>
+      <c r="AM21" s="16" t="n"/>
+      <c r="AN21" s="25" t="n"/>
+      <c r="AO21" s="48" t="n"/>
+      <c r="AP21" s="23" t="n"/>
+      <c r="AQ21" s="15" t="n"/>
+      <c r="AR21" s="15" t="n"/>
+      <c r="AS21" s="16" t="n"/>
+      <c r="AT21" s="25" t="n"/>
+      <c r="AU21" s="26" t="n"/>
+    </row>
+    <row r="22" ht="25.5" customHeight="1" s="71">
+      <c r="D22" s="18" t="n"/>
+      <c r="J22" s="15" t="n"/>
+      <c r="K22" s="15" t="n"/>
+      <c r="L22" s="16" t="n"/>
+      <c r="R22" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="S22" s="15" t="n"/>
+      <c r="T22" s="15" t="n"/>
+      <c r="U22" s="16" t="n"/>
+      <c r="X22" s="21" t="n"/>
+      <c r="Y22" s="15" t="n"/>
+      <c r="Z22" s="15" t="n"/>
+      <c r="AA22" s="16" t="n"/>
+      <c r="AD22" s="22" t="n"/>
+      <c r="AE22" s="15" t="n"/>
+      <c r="AF22" s="15" t="n"/>
+      <c r="AG22" s="16" t="n"/>
+      <c r="AH22" s="48" t="n"/>
+      <c r="AI22" s="48" t="n"/>
+      <c r="AJ22" s="23" t="n"/>
+      <c r="AK22" s="15" t="n"/>
+      <c r="AL22" s="15" t="n"/>
+      <c r="AM22" s="16" t="n"/>
+      <c r="AP22" s="23" t="n"/>
+      <c r="AQ22" s="15" t="n"/>
+      <c r="AR22" s="15" t="n"/>
+      <c r="AS22" s="16" t="n"/>
+    </row>
+    <row r="23" s="71">
+      <c r="D23" s="18" t="n"/>
+      <c r="J23" s="15" t="n"/>
+      <c r="K23" s="15" t="n"/>
+      <c r="L23" s="16" t="n"/>
+      <c r="R23" s="19" t="n">
+        <v>300</v>
+      </c>
+      <c r="S23" s="15" t="n"/>
+      <c r="T23" s="15" t="n"/>
+      <c r="U23" s="16" t="n"/>
+      <c r="X23" s="21" t="n"/>
+      <c r="Y23" s="15" t="n"/>
+      <c r="Z23" s="15" t="n"/>
+      <c r="AA23" s="16" t="n"/>
+      <c r="AD23" s="22" t="n"/>
+      <c r="AE23" s="15" t="n"/>
+      <c r="AF23" s="15" t="n"/>
+      <c r="AG23" s="16" t="n"/>
+      <c r="AH23" s="48" t="n"/>
+      <c r="AI23" s="48" t="n"/>
+      <c r="AJ23" s="23" t="n"/>
+      <c r="AK23" s="15" t="n"/>
+      <c r="AL23" s="15" t="n"/>
+      <c r="AM23" s="16" t="n"/>
+      <c r="AP23" s="23" t="n"/>
+      <c r="AQ23" s="15" t="n"/>
+      <c r="AR23" s="15" t="n"/>
+      <c r="AS23" s="16" t="n"/>
+    </row>
+    <row r="24" ht="6.75" customHeight="1" s="71">
+      <c r="A24" s="27" t="n"/>
+      <c r="B24" s="27" t="n"/>
+      <c r="C24" s="27" t="n"/>
+      <c r="D24" s="27" t="n"/>
+      <c r="E24" s="27" t="n"/>
+      <c r="F24" s="27" t="n"/>
+      <c r="G24" s="27" t="n"/>
+      <c r="H24" s="35" t="n"/>
+      <c r="I24" s="35" t="n"/>
+      <c r="J24" s="36" t="n"/>
+      <c r="K24" s="36" t="n"/>
+      <c r="L24" s="36" t="n"/>
+      <c r="M24" s="35" t="n"/>
+      <c r="N24" s="30" t="n"/>
+      <c r="O24" s="30" t="n"/>
+      <c r="P24" s="30" t="n"/>
+      <c r="Q24" s="30" t="n"/>
+      <c r="R24" s="35" t="n"/>
+      <c r="S24" s="35" t="n"/>
+      <c r="T24" s="35" t="n"/>
+      <c r="U24" s="35" t="n"/>
+      <c r="V24" s="35" t="n"/>
+      <c r="W24" s="35" t="n"/>
+      <c r="X24" s="31" t="n"/>
+      <c r="Y24" s="35" t="n"/>
+      <c r="Z24" s="35" t="n"/>
+      <c r="AA24" s="36" t="n"/>
+      <c r="AB24" s="35" t="n"/>
+      <c r="AC24" s="35" t="n"/>
+      <c r="AD24" s="32" t="n"/>
+      <c r="AE24" s="35" t="n"/>
+      <c r="AF24" s="35" t="n"/>
+      <c r="AG24" s="36" t="n"/>
+      <c r="AH24" s="35" t="n"/>
+      <c r="AI24" s="35" t="n"/>
+      <c r="AJ24" s="34" t="n"/>
+      <c r="AK24" s="35" t="n"/>
+      <c r="AL24" s="35" t="n"/>
+      <c r="AM24" s="36" t="n"/>
+      <c r="AN24" s="35" t="n"/>
+      <c r="AO24" s="35" t="n"/>
+      <c r="AP24" s="34" t="n"/>
+      <c r="AQ24" s="35" t="n"/>
+      <c r="AR24" s="35" t="n"/>
+      <c r="AS24" s="36" t="n"/>
+      <c r="AT24" s="35" t="n"/>
+      <c r="AU24" s="35" t="n"/>
+    </row>
+    <row r="25" ht="24" customHeight="1" s="71">
+      <c r="A25" s="10">
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S7bf6b53d95ef4513a8cbc9bfe0979eed6.jpg")</f>
+        <v/>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>Trailer Wheel Bearing Protectors Stainless Steel Hub Caps Dust Covers …</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>AliExpress: US $16.12. Vår räkning: landad ca 232 kr, tänkt butikspris 599 kr. Originaltitel: 2Pcs Trailer Wheel Bearing Protectors Stainless Steel Hub Caps Dust Covers Replacement 1.98 Inch for Rv Utility Boat Trailers</t>
+        </is>
+      </c>
+      <c r="H25" s="13" t="n"/>
+      <c r="I25" s="14" t="inlineStr">
+        <is>
+          <t>SWEDEN</t>
+        </is>
+      </c>
+      <c r="J25" s="15" t="n"/>
+      <c r="K25" s="15" t="n"/>
+      <c r="L25" s="16" t="n"/>
+      <c r="M25" s="14" t="n"/>
+      <c r="N25" s="17" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.com/item/1005013066657447.html</t>
+        </is>
+      </c>
+      <c r="Q25" s="18" t="n"/>
+      <c r="R25" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="S25" s="15" t="n"/>
+      <c r="T25" s="15" t="n"/>
+      <c r="U25" s="16" t="n"/>
+      <c r="V25" s="48" t="n"/>
+      <c r="W25" s="48" t="n"/>
+      <c r="X25" s="21" t="n"/>
+      <c r="Y25" s="15" t="n"/>
+      <c r="Z25" s="15" t="n"/>
+      <c r="AA25" s="16" t="n"/>
+      <c r="AB25" s="48" t="n"/>
+      <c r="AC25" s="48" t="n"/>
+      <c r="AD25" s="22" t="n"/>
+      <c r="AE25" s="15" t="n"/>
+      <c r="AF25" s="15" t="n"/>
+      <c r="AG25" s="16" t="n"/>
+      <c r="AH25" s="48" t="n"/>
+      <c r="AI25" s="48" t="n"/>
+      <c r="AJ25" s="23" t="n"/>
+      <c r="AK25" s="15" t="n"/>
+      <c r="AL25" s="15" t="n"/>
+      <c r="AM25" s="16" t="n"/>
+      <c r="AN25" s="25" t="n"/>
+      <c r="AO25" s="48" t="n"/>
+      <c r="AP25" s="23" t="n"/>
+      <c r="AQ25" s="15" t="n"/>
+      <c r="AR25" s="15" t="n"/>
+      <c r="AS25" s="16" t="n"/>
+      <c r="AT25" s="25" t="n"/>
+      <c r="AU25" s="26" t="n"/>
+    </row>
+    <row r="26" ht="25.5" customHeight="1" s="71">
+      <c r="D26" s="18" t="n"/>
+      <c r="J26" s="15" t="n"/>
+      <c r="K26" s="15" t="n"/>
+      <c r="L26" s="16" t="n"/>
+      <c r="R26" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="S26" s="15" t="n"/>
+      <c r="T26" s="15" t="n"/>
+      <c r="U26" s="16" t="n"/>
+      <c r="X26" s="21" t="n"/>
+      <c r="Y26" s="15" t="n"/>
+      <c r="Z26" s="15" t="n"/>
+      <c r="AA26" s="16" t="n"/>
+      <c r="AD26" s="22" t="n"/>
+      <c r="AE26" s="15" t="n"/>
+      <c r="AF26" s="15" t="n"/>
+      <c r="AG26" s="16" t="n"/>
+      <c r="AH26" s="48" t="n"/>
+      <c r="AI26" s="48" t="n"/>
+      <c r="AJ26" s="23" t="n"/>
+      <c r="AK26" s="15" t="n"/>
+      <c r="AL26" s="15" t="n"/>
+      <c r="AM26" s="16" t="n"/>
+      <c r="AP26" s="23" t="n"/>
+      <c r="AQ26" s="15" t="n"/>
+      <c r="AR26" s="15" t="n"/>
+      <c r="AS26" s="16" t="n"/>
+    </row>
+    <row r="27" s="71">
+      <c r="D27" s="18" t="n"/>
+      <c r="J27" s="15" t="n"/>
+      <c r="K27" s="15" t="n"/>
+      <c r="L27" s="16" t="n"/>
+      <c r="R27" s="19" t="n">
+        <v>300</v>
+      </c>
+      <c r="S27" s="15" t="n"/>
+      <c r="T27" s="15" t="n"/>
+      <c r="U27" s="16" t="n"/>
+      <c r="X27" s="21" t="n"/>
+      <c r="Y27" s="15" t="n"/>
+      <c r="Z27" s="15" t="n"/>
+      <c r="AA27" s="16" t="n"/>
+      <c r="AD27" s="22" t="n"/>
+      <c r="AE27" s="15" t="n"/>
+      <c r="AF27" s="15" t="n"/>
+      <c r="AG27" s="16" t="n"/>
+      <c r="AH27" s="48" t="n"/>
+      <c r="AI27" s="48" t="n"/>
+      <c r="AJ27" s="23" t="n"/>
+      <c r="AK27" s="15" t="n"/>
+      <c r="AL27" s="15" t="n"/>
+      <c r="AM27" s="16" t="n"/>
+      <c r="AP27" s="23" t="n"/>
+      <c r="AQ27" s="15" t="n"/>
+      <c r="AR27" s="15" t="n"/>
+      <c r="AS27" s="16" t="n"/>
+    </row>
+    <row r="28" ht="6.75" customHeight="1" s="71">
+      <c r="A28" s="27" t="n"/>
+      <c r="B28" s="27" t="n"/>
+      <c r="C28" s="27" t="n"/>
+      <c r="D28" s="27" t="n"/>
+      <c r="E28" s="27" t="n"/>
+      <c r="F28" s="27" t="n"/>
+      <c r="G28" s="27" t="n"/>
+      <c r="H28" s="35" t="n"/>
+      <c r="I28" s="35" t="n"/>
+      <c r="J28" s="36" t="n"/>
+      <c r="K28" s="36" t="n"/>
+      <c r="L28" s="36" t="n"/>
+      <c r="M28" s="35" t="n"/>
+      <c r="N28" s="30" t="n"/>
+      <c r="O28" s="30" t="n"/>
+      <c r="P28" s="30" t="n"/>
+      <c r="Q28" s="30" t="n"/>
+      <c r="R28" s="35" t="n"/>
+      <c r="S28" s="35" t="n"/>
+      <c r="T28" s="35" t="n"/>
+      <c r="U28" s="35" t="n"/>
+      <c r="V28" s="35" t="n"/>
+      <c r="W28" s="35" t="n"/>
+      <c r="X28" s="31" t="n"/>
+      <c r="Y28" s="35" t="n"/>
+      <c r="Z28" s="35" t="n"/>
+      <c r="AA28" s="36" t="n"/>
+      <c r="AB28" s="35" t="n"/>
+      <c r="AC28" s="35" t="n"/>
+      <c r="AD28" s="32" t="n"/>
+      <c r="AE28" s="35" t="n"/>
+      <c r="AF28" s="35" t="n"/>
+      <c r="AG28" s="36" t="n"/>
+      <c r="AH28" s="35" t="n"/>
+      <c r="AI28" s="35" t="n"/>
+      <c r="AJ28" s="34" t="n"/>
+      <c r="AK28" s="35" t="n"/>
+      <c r="AL28" s="35" t="n"/>
+      <c r="AM28" s="36" t="n"/>
+      <c r="AN28" s="35" t="n"/>
+      <c r="AO28" s="35" t="n"/>
+      <c r="AP28" s="34" t="n"/>
+      <c r="AQ28" s="35" t="n"/>
+      <c r="AR28" s="35" t="n"/>
+      <c r="AS28" s="36" t="n"/>
+      <c r="AT28" s="35" t="n"/>
+      <c r="AU28" s="35" t="n"/>
+    </row>
+    <row r="29" ht="24" customHeight="1" s="71">
+      <c r="A29" s="10">
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S460c4c1b988e42a1b514fe6616d50baae.png")</f>
+        <v/>
+      </c>
+      <c r="D29" s="18" t="inlineStr">
+        <is>
+          <t>Car Washer Mop Foam Wash Brush Double Brush Head Roof Window Cleaning …</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>AliExpress: US $12.88. Vår räkning: landad ca 186 kr, tänkt butikspris 499 kr. Originaltitel: Car Washer Mop Foam Wash Brush Double Brush Head Roof Window Cleaning Maintenance Three-Section Telescopic Mop Car Accessories</t>
+        </is>
+      </c>
+      <c r="H29" s="13" t="n"/>
+      <c r="I29" s="14" t="inlineStr">
+        <is>
+          <t>SWEDEN</t>
+        </is>
+      </c>
+      <c r="J29" s="15" t="n"/>
+      <c r="K29" s="15" t="n"/>
+      <c r="L29" s="16" t="n"/>
+      <c r="M29" s="14" t="n"/>
+      <c r="N29" s="17" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.com/item/1005007159566417.html</t>
+        </is>
+      </c>
+      <c r="Q29" s="18" t="n"/>
+      <c r="R29" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="S29" s="15" t="n"/>
+      <c r="T29" s="15" t="n"/>
+      <c r="U29" s="16" t="n"/>
+      <c r="V29" s="48" t="n"/>
+      <c r="W29" s="48" t="n"/>
+      <c r="X29" s="21" t="n"/>
+      <c r="Y29" s="15" t="n"/>
+      <c r="Z29" s="15" t="n"/>
+      <c r="AA29" s="16" t="n"/>
+      <c r="AB29" s="48" t="n"/>
+      <c r="AC29" s="48" t="n"/>
+      <c r="AD29" s="22" t="n"/>
+      <c r="AE29" s="15" t="n"/>
+      <c r="AF29" s="15" t="n"/>
+      <c r="AG29" s="16" t="n"/>
+      <c r="AH29" s="48" t="n"/>
+      <c r="AI29" s="48" t="n"/>
+      <c r="AJ29" s="23" t="n"/>
+      <c r="AK29" s="15" t="n"/>
+      <c r="AL29" s="15" t="n"/>
+      <c r="AM29" s="16" t="n"/>
+      <c r="AN29" s="25" t="n"/>
+      <c r="AO29" s="48" t="n"/>
+      <c r="AP29" s="23" t="n"/>
+      <c r="AQ29" s="15" t="n"/>
+      <c r="AR29" s="15" t="n"/>
+      <c r="AS29" s="16" t="n"/>
+      <c r="AT29" s="25" t="n"/>
+      <c r="AU29" s="26" t="n"/>
+    </row>
+    <row r="30" ht="25.5" customHeight="1" s="71">
+      <c r="D30" s="18" t="n"/>
+      <c r="J30" s="15" t="n"/>
+      <c r="K30" s="15" t="n"/>
+      <c r="L30" s="16" t="n"/>
+      <c r="R30" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="S30" s="15" t="n"/>
+      <c r="T30" s="15" t="n"/>
+      <c r="U30" s="16" t="n"/>
+      <c r="X30" s="21" t="n"/>
+      <c r="Y30" s="15" t="n"/>
+      <c r="Z30" s="15" t="n"/>
+      <c r="AA30" s="16" t="n"/>
+      <c r="AD30" s="22" t="n"/>
+      <c r="AE30" s="15" t="n"/>
+      <c r="AF30" s="15" t="n"/>
+      <c r="AG30" s="16" t="n"/>
+      <c r="AH30" s="48" t="n"/>
+      <c r="AI30" s="48" t="n"/>
+      <c r="AJ30" s="23" t="n"/>
+      <c r="AK30" s="15" t="n"/>
+      <c r="AL30" s="15" t="n"/>
+      <c r="AM30" s="16" t="n"/>
+      <c r="AP30" s="23" t="n"/>
+      <c r="AQ30" s="15" t="n"/>
+      <c r="AR30" s="15" t="n"/>
+      <c r="AS30" s="16" t="n"/>
+    </row>
+    <row r="31" s="71">
+      <c r="D31" s="18" t="n"/>
+      <c r="J31" s="15" t="n"/>
+      <c r="K31" s="15" t="n"/>
+      <c r="L31" s="16" t="n"/>
+      <c r="R31" s="19" t="n">
+        <v>300</v>
+      </c>
+      <c r="S31" s="15" t="n"/>
+      <c r="T31" s="15" t="n"/>
+      <c r="U31" s="16" t="n"/>
+      <c r="X31" s="21" t="n"/>
+      <c r="Y31" s="15" t="n"/>
+      <c r="Z31" s="15" t="n"/>
+      <c r="AA31" s="16" t="n"/>
+      <c r="AD31" s="22" t="n"/>
+      <c r="AE31" s="15" t="n"/>
+      <c r="AF31" s="15" t="n"/>
+      <c r="AG31" s="16" t="n"/>
+      <c r="AH31" s="48" t="n"/>
+      <c r="AI31" s="48" t="n"/>
+      <c r="AJ31" s="23" t="n"/>
+      <c r="AK31" s="15" t="n"/>
+      <c r="AL31" s="15" t="n"/>
+      <c r="AM31" s="16" t="n"/>
+      <c r="AP31" s="23" t="n"/>
+      <c r="AQ31" s="15" t="n"/>
+      <c r="AR31" s="15" t="n"/>
+      <c r="AS31" s="16" t="n"/>
+    </row>
+    <row r="32" ht="6.75" customHeight="1" s="71">
+      <c r="A32" s="27" t="n"/>
+      <c r="B32" s="27" t="n"/>
+      <c r="C32" s="27" t="n"/>
+      <c r="D32" s="27" t="n"/>
+      <c r="E32" s="27" t="n"/>
+      <c r="F32" s="27" t="n"/>
+      <c r="G32" s="27" t="n"/>
+      <c r="H32" s="35" t="n"/>
+      <c r="I32" s="35" t="n"/>
+      <c r="J32" s="36" t="n"/>
+      <c r="K32" s="36" t="n"/>
+      <c r="L32" s="36" t="n"/>
+      <c r="M32" s="35" t="n"/>
+      <c r="N32" s="30" t="n"/>
+      <c r="O32" s="30" t="n"/>
+      <c r="P32" s="30" t="n"/>
+      <c r="Q32" s="30" t="n"/>
+      <c r="R32" s="35" t="n"/>
+      <c r="S32" s="35" t="n"/>
+      <c r="T32" s="35" t="n"/>
+      <c r="U32" s="35" t="n"/>
+      <c r="V32" s="35" t="n"/>
+      <c r="W32" s="35" t="n"/>
+      <c r="X32" s="31" t="n"/>
+      <c r="Y32" s="35" t="n"/>
+      <c r="Z32" s="35" t="n"/>
+      <c r="AA32" s="36" t="n"/>
+      <c r="AB32" s="35" t="n"/>
+      <c r="AC32" s="35" t="n"/>
+      <c r="AD32" s="32" t="n"/>
+      <c r="AE32" s="35" t="n"/>
+      <c r="AF32" s="35" t="n"/>
+      <c r="AG32" s="36" t="n"/>
+      <c r="AH32" s="35" t="n"/>
+      <c r="AI32" s="35" t="n"/>
+      <c r="AJ32" s="34" t="n"/>
+      <c r="AK32" s="35" t="n"/>
+      <c r="AL32" s="35" t="n"/>
+      <c r="AM32" s="36" t="n"/>
+      <c r="AN32" s="35" t="n"/>
+      <c r="AO32" s="35" t="n"/>
+      <c r="AP32" s="34" t="n"/>
+      <c r="AQ32" s="35" t="n"/>
+      <c r="AR32" s="35" t="n"/>
+      <c r="AS32" s="36" t="n"/>
+      <c r="AT32" s="35" t="n"/>
+      <c r="AU32" s="35" t="n"/>
+    </row>
+    <row r="33" ht="24" customHeight="1" s="71">
+      <c r="A33" s="10">
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S46f2a551fb2044e6b96fc5ce0181a075w.png")</f>
+        <v/>
+      </c>
+      <c r="D33" s="18" t="inlineStr">
+        <is>
+          <t>New 110dB Door And Window Vibration Alarm Wireless Anti-Theft Alarm Wi…</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>AliExpress: US $13.23. Vår räkning: landad ca 191 kr, tänkt butikspris 499 kr. Originaltitel: New 110dB Door And Window Vibration Alarm Wireless Anti-Theft  Alarm With Remote Control Home Bicycle Security Burglar Alarm</t>
+        </is>
+      </c>
+      <c r="H33" s="13" t="n"/>
+      <c r="I33" s="14" t="inlineStr">
+        <is>
+          <t>SWEDEN</t>
+        </is>
+      </c>
+      <c r="J33" s="15" t="n"/>
+      <c r="K33" s="15" t="n"/>
+      <c r="L33" s="16" t="n"/>
+      <c r="M33" s="14" t="n"/>
+      <c r="N33" s="17" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.com/item/1005007345104914.html</t>
+        </is>
+      </c>
+      <c r="Q33" s="18" t="n"/>
+      <c r="R33" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="S33" s="15" t="n"/>
+      <c r="T33" s="15" t="n"/>
+      <c r="U33" s="16" t="n"/>
+      <c r="V33" s="48" t="n"/>
+      <c r="W33" s="48" t="n"/>
+      <c r="X33" s="21" t="n"/>
+      <c r="Y33" s="15" t="n"/>
+      <c r="Z33" s="15" t="n"/>
+      <c r="AA33" s="16" t="n"/>
+      <c r="AB33" s="48" t="n"/>
+      <c r="AC33" s="48" t="n"/>
+      <c r="AD33" s="22" t="n"/>
+      <c r="AE33" s="15" t="n"/>
+      <c r="AF33" s="15" t="n"/>
+      <c r="AG33" s="16" t="n"/>
+      <c r="AH33" s="48" t="n"/>
+      <c r="AI33" s="48" t="n"/>
+      <c r="AJ33" s="23" t="n"/>
+      <c r="AK33" s="15" t="n"/>
+      <c r="AL33" s="15" t="n"/>
+      <c r="AM33" s="16" t="n"/>
+      <c r="AN33" s="25" t="n"/>
+      <c r="AO33" s="48" t="n"/>
+      <c r="AP33" s="23" t="n"/>
+      <c r="AQ33" s="15" t="n"/>
+      <c r="AR33" s="15" t="n"/>
+      <c r="AS33" s="16" t="n"/>
+      <c r="AT33" s="25" t="n"/>
+      <c r="AU33" s="26" t="n"/>
+    </row>
+    <row r="34" ht="25.5" customHeight="1" s="71">
+      <c r="D34" s="18" t="n"/>
+      <c r="J34" s="15" t="n"/>
+      <c r="K34" s="15" t="n"/>
+      <c r="L34" s="16" t="n"/>
+      <c r="R34" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="S34" s="15" t="n"/>
+      <c r="T34" s="15" t="n"/>
+      <c r="U34" s="16" t="n"/>
+      <c r="X34" s="21" t="n"/>
+      <c r="Y34" s="15" t="n"/>
+      <c r="Z34" s="15" t="n"/>
+      <c r="AA34" s="16" t="n"/>
+      <c r="AD34" s="22" t="n"/>
+      <c r="AE34" s="15" t="n"/>
+      <c r="AF34" s="15" t="n"/>
+      <c r="AG34" s="16" t="n"/>
+      <c r="AH34" s="48" t="n"/>
+      <c r="AI34" s="48" t="n"/>
+      <c r="AJ34" s="23" t="n"/>
+      <c r="AK34" s="15" t="n"/>
+      <c r="AL34" s="15" t="n"/>
+      <c r="AM34" s="16" t="n"/>
+      <c r="AP34" s="23" t="n"/>
+      <c r="AQ34" s="15" t="n"/>
+      <c r="AR34" s="15" t="n"/>
+      <c r="AS34" s="16" t="n"/>
+    </row>
+    <row r="35" s="71">
+      <c r="D35" s="18" t="n"/>
+      <c r="J35" s="15" t="n"/>
+      <c r="K35" s="15" t="n"/>
+      <c r="L35" s="16" t="n"/>
+      <c r="R35" s="19" t="n">
+        <v>300</v>
+      </c>
+      <c r="S35" s="15" t="n"/>
+      <c r="T35" s="15" t="n"/>
+      <c r="U35" s="16" t="n"/>
+      <c r="X35" s="21" t="n"/>
+      <c r="Y35" s="15" t="n"/>
+      <c r="Z35" s="15" t="n"/>
+      <c r="AA35" s="16" t="n"/>
+      <c r="AD35" s="22" t="n"/>
+      <c r="AE35" s="15" t="n"/>
+      <c r="AF35" s="15" t="n"/>
+      <c r="AG35" s="16" t="n"/>
+      <c r="AH35" s="48" t="n"/>
+      <c r="AI35" s="48" t="n"/>
+      <c r="AJ35" s="23" t="n"/>
+      <c r="AK35" s="15" t="n"/>
+      <c r="AL35" s="15" t="n"/>
+      <c r="AM35" s="16" t="n"/>
+      <c r="AP35" s="23" t="n"/>
+      <c r="AQ35" s="15" t="n"/>
+      <c r="AR35" s="15" t="n"/>
+      <c r="AS35" s="16" t="n"/>
+    </row>
+    <row r="36" ht="6.75" customHeight="1" s="71">
+      <c r="A36" s="27" t="n"/>
+      <c r="B36" s="27" t="n"/>
+      <c r="C36" s="27" t="n"/>
+      <c r="D36" s="27" t="n"/>
+      <c r="E36" s="27" t="n"/>
+      <c r="F36" s="27" t="n"/>
+      <c r="G36" s="27" t="n"/>
+      <c r="H36" s="35" t="n"/>
+      <c r="I36" s="35" t="n"/>
+      <c r="J36" s="36" t="n"/>
+      <c r="K36" s="36" t="n"/>
+      <c r="L36" s="36" t="n"/>
+      <c r="M36" s="35" t="n"/>
+      <c r="N36" s="30" t="n"/>
+      <c r="O36" s="30" t="n"/>
+      <c r="P36" s="30" t="n"/>
+      <c r="Q36" s="30" t="n"/>
+      <c r="R36" s="35" t="n"/>
+      <c r="S36" s="35" t="n"/>
+      <c r="T36" s="35" t="n"/>
+      <c r="U36" s="35" t="n"/>
+      <c r="V36" s="35" t="n"/>
+      <c r="W36" s="35" t="n"/>
+      <c r="X36" s="31" t="n"/>
+      <c r="Y36" s="35" t="n"/>
+      <c r="Z36" s="35" t="n"/>
+      <c r="AA36" s="36" t="n"/>
+      <c r="AB36" s="35" t="n"/>
+      <c r="AC36" s="35" t="n"/>
+      <c r="AD36" s="32" t="n"/>
+      <c r="AE36" s="35" t="n"/>
+      <c r="AF36" s="35" t="n"/>
+      <c r="AG36" s="36" t="n"/>
+      <c r="AH36" s="35" t="n"/>
+      <c r="AI36" s="35" t="n"/>
+      <c r="AJ36" s="34" t="n"/>
+      <c r="AK36" s="35" t="n"/>
+      <c r="AL36" s="35" t="n"/>
+      <c r="AM36" s="36" t="n"/>
+      <c r="AN36" s="35" t="n"/>
+      <c r="AO36" s="35" t="n"/>
+      <c r="AP36" s="34" t="n"/>
+      <c r="AQ36" s="35" t="n"/>
+      <c r="AR36" s="35" t="n"/>
+      <c r="AS36" s="36" t="n"/>
+      <c r="AT36" s="35" t="n"/>
+      <c r="AU36" s="35" t="n"/>
+    </row>
+    <row r="37" ht="24" customHeight="1" s="71">
+      <c r="A37" s="10">
+        <f>IMAGE("https://ae-pic-a1.aliexpress-media.com/kf/S8256719988c545fa8eae78575fd2166fC.jpg")</f>
+        <v/>
+      </c>
+      <c r="D37" s="18" t="inlineStr">
+        <is>
+          <t>COB LED Work Light Rechargeable Outdoor Emergency Lighting Led Work Li…</t>
+        </is>
+      </c>
+      <c r="E37" s="12" t="inlineStr">
+        <is>
+          <t>AliExpress: US $16.01. Vår räkning: landad ca 231 kr, tänkt butikspris 599 kr. Originaltitel: COB LED Work Light Rechargeable Outdoor Emergency Lighting Led Work Light with 360° Swivel Hose,Magnetic,Hanging Hook Car Repair</t>
+        </is>
+      </c>
+      <c r="H37" s="13" t="n"/>
+      <c r="I37" s="14" t="inlineStr">
+        <is>
+          <t>SWEDEN</t>
+        </is>
+      </c>
+      <c r="J37" s="15" t="n"/>
+      <c r="K37" s="15" t="n"/>
+      <c r="L37" s="16" t="n"/>
+      <c r="M37" s="14" t="n"/>
+      <c r="N37" s="17" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.com/item/1005012197673762.html</t>
+        </is>
+      </c>
+      <c r="Q37" s="18" t="n"/>
+      <c r="R37" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="S37" s="15" t="n"/>
+      <c r="T37" s="15" t="n"/>
+      <c r="U37" s="16" t="n"/>
+      <c r="V37" s="48" t="n"/>
+      <c r="W37" s="48" t="n"/>
+      <c r="X37" s="21" t="n"/>
+      <c r="Y37" s="15" t="n"/>
+      <c r="Z37" s="15" t="n"/>
+      <c r="AA37" s="16" t="n"/>
+      <c r="AB37" s="48" t="n"/>
+      <c r="AC37" s="48" t="n"/>
+      <c r="AD37" s="22" t="n"/>
+      <c r="AE37" s="15" t="n"/>
+      <c r="AF37" s="15" t="n"/>
+      <c r="AG37" s="16" t="n"/>
+      <c r="AH37" s="48" t="n"/>
+      <c r="AI37" s="48" t="n"/>
+      <c r="AJ37" s="23" t="n"/>
+      <c r="AK37" s="15" t="n"/>
+      <c r="AL37" s="15" t="n"/>
+      <c r="AM37" s="16" t="n"/>
+      <c r="AN37" s="25" t="n"/>
+      <c r="AO37" s="48" t="n"/>
+      <c r="AP37" s="23" t="n"/>
+      <c r="AQ37" s="15" t="n"/>
+      <c r="AR37" s="15" t="n"/>
+      <c r="AS37" s="16" t="n"/>
+      <c r="AT37" s="25" t="n"/>
+      <c r="AU37" s="26" t="n"/>
+    </row>
+    <row r="38" ht="25.5" customHeight="1" s="71">
+      <c r="D38" s="18" t="n"/>
+      <c r="J38" s="15" t="n"/>
+      <c r="K38" s="15" t="n"/>
+      <c r="L38" s="16" t="n"/>
+      <c r="R38" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="S38" s="15" t="n"/>
+      <c r="T38" s="15" t="n"/>
+      <c r="U38" s="16" t="n"/>
+      <c r="X38" s="21" t="n"/>
+      <c r="Y38" s="15" t="n"/>
+      <c r="Z38" s="15" t="n"/>
+      <c r="AA38" s="16" t="n"/>
+      <c r="AD38" s="22" t="n"/>
+      <c r="AE38" s="15" t="n"/>
+      <c r="AF38" s="15" t="n"/>
+      <c r="AG38" s="16" t="n"/>
+      <c r="AH38" s="48" t="n"/>
+      <c r="AI38" s="48" t="n"/>
+      <c r="AJ38" s="23" t="n"/>
+      <c r="AK38" s="15" t="n"/>
+      <c r="AL38" s="15" t="n"/>
+      <c r="AM38" s="16" t="n"/>
+      <c r="AP38" s="23" t="n"/>
+      <c r="AQ38" s="15" t="n"/>
+      <c r="AR38" s="15" t="n"/>
+      <c r="AS38" s="16" t="n"/>
+    </row>
+    <row r="39" s="71">
+      <c r="D39" s="18" t="n"/>
+      <c r="J39" s="15" t="n"/>
+      <c r="K39" s="15" t="n"/>
+      <c r="L39" s="16" t="n"/>
+      <c r="R39" s="19" t="n">
+        <v>300</v>
+      </c>
+      <c r="S39" s="15" t="n"/>
+      <c r="T39" s="15" t="n"/>
+      <c r="U39" s="16" t="n"/>
+      <c r="X39" s="21" t="n"/>
+      <c r="Y39" s="15" t="n"/>
+      <c r="Z39" s="15" t="n"/>
+      <c r="AA39" s="16" t="n"/>
+      <c r="AD39" s="22" t="n"/>
+      <c r="AE39" s="15" t="n"/>
+      <c r="AF39" s="15" t="n"/>
+      <c r="AG39" s="16" t="n"/>
+      <c r="AH39" s="48" t="n"/>
+      <c r="AI39" s="48" t="n"/>
+      <c r="AJ39" s="23" t="n"/>
+      <c r="AK39" s="15" t="n"/>
+      <c r="AL39" s="15" t="n"/>
+      <c r="AM39" s="16" t="n"/>
+      <c r="AP39" s="23" t="n"/>
+      <c r="AQ39" s="15" t="n"/>
+      <c r="AR39" s="15" t="n"/>
+      <c r="AS39" s="16" t="n"/>
+    </row>
+    <row r="40" ht="6.75" customHeight="1" s="71">
+      <c r="A40" s="27" t="n"/>
+      <c r="B40" s="27" t="n"/>
+      <c r="C40" s="27" t="n"/>
+      <c r="D40" s="27" t="n"/>
+      <c r="E40" s="27" t="n"/>
+      <c r="F40" s="27" t="n"/>
+      <c r="G40" s="27" t="n"/>
+      <c r="H40" s="35" t="n"/>
+      <c r="I40" s="35" t="n"/>
+      <c r="J40" s="36" t="n"/>
+      <c r="K40" s="36" t="n"/>
+      <c r="L40" s="36" t="n"/>
+      <c r="M40" s="35" t="n"/>
+      <c r="N40" s="30" t="n"/>
+      <c r="O40" s="30" t="n"/>
+      <c r="P40" s="30" t="n"/>
+      <c r="Q40" s="30" t="n"/>
+      <c r="R40" s="35" t="n"/>
+      <c r="S40" s="35" t="n"/>
+      <c r="T40" s="35" t="n"/>
+      <c r="U40" s="35" t="n"/>
+      <c r="V40" s="35" t="n"/>
+      <c r="W40" s="35" t="n"/>
+      <c r="X40" s="31" t="n"/>
+      <c r="Y40" s="35" t="n"/>
+      <c r="Z40" s="35" t="n"/>
+      <c r="AA40" s="36" t="n"/>
+      <c r="AB40" s="35" t="n"/>
+      <c r="AC40" s="35" t="n"/>
+      <c r="AD40" s="32" t="n"/>
+      <c r="AE40" s="35" t="n"/>
+      <c r="AF40" s="35" t="n"/>
+      <c r="AG40" s="36" t="n"/>
+      <c r="AH40" s="35" t="n"/>
+      <c r="AI40" s="35" t="n"/>
+      <c r="AJ40" s="34" t="n"/>
+      <c r="AK40" s="35" t="n"/>
+      <c r="AL40" s="35" t="n"/>
+      <c r="AM40" s="36" t="n"/>
+      <c r="AN40" s="35" t="n"/>
+      <c r="AO40" s="35" t="n"/>
+      <c r="AP40" s="34" t="n"/>
+      <c r="AQ40" s="35" t="n"/>
+      <c r="AR40" s="35" t="n"/>
+      <c r="AS40" s="36" t="n"/>
+      <c r="AT40" s="35" t="n"/>
+      <c r="AU40" s="35" t="n"/>
+    </row>
     <row r="41" ht="15.75" customHeight="1" s="71"/>
     <row r="42" ht="15.75" customHeight="1" s="71"/>
     <row r="43" ht="15.75" customHeight="1" s="71"/>
@@ -2529,46 +3543,91 @@
     <row r="999" ht="15.75" customHeight="1" s="71"/>
     <row r="1000" ht="15.75" customHeight="1" s="71"/>
   </sheetData>
-  <mergeCells count="38">
+  <mergeCells count="80">
+    <mergeCell ref="E5:G7"/>
+    <mergeCell ref="H17:H19"/>
+    <mergeCell ref="M21:M23"/>
+    <mergeCell ref="L3:L4"/>
+    <mergeCell ref="N5:P7"/>
+    <mergeCell ref="N33:P35"/>
+    <mergeCell ref="A37:C39"/>
+    <mergeCell ref="R3:W3"/>
+    <mergeCell ref="A21:C23"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="H5:H7"/>
+    <mergeCell ref="A29:C31"/>
+    <mergeCell ref="M5:M7"/>
+    <mergeCell ref="H29:H31"/>
+    <mergeCell ref="A13:C15"/>
+    <mergeCell ref="Q33:Q35"/>
+    <mergeCell ref="AD3:AI3"/>
+    <mergeCell ref="E25:G27"/>
+    <mergeCell ref="AP3:AU3"/>
+    <mergeCell ref="H21:H23"/>
+    <mergeCell ref="M25:M27"/>
+    <mergeCell ref="Q3:Q4"/>
+    <mergeCell ref="E17:G19"/>
+    <mergeCell ref="I37:I39"/>
+    <mergeCell ref="Q9:Q11"/>
+    <mergeCell ref="I29:I31"/>
+    <mergeCell ref="I13:I15"/>
+    <mergeCell ref="M29:M31"/>
+    <mergeCell ref="A1:AO1"/>
+    <mergeCell ref="H33:H35"/>
+    <mergeCell ref="N17:P19"/>
+    <mergeCell ref="A5:C7"/>
+    <mergeCell ref="N3:P4"/>
+    <mergeCell ref="H25:H27"/>
+    <mergeCell ref="N9:P11"/>
+    <mergeCell ref="E21:G23"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="I25:I27"/>
+    <mergeCell ref="I33:I35"/>
     <mergeCell ref="I5:I7"/>
-    <mergeCell ref="E5:G7"/>
-    <mergeCell ref="Q9:Q11"/>
-    <mergeCell ref="L3:L4"/>
-    <mergeCell ref="E13:G15"/>
+    <mergeCell ref="I17:I19"/>
+    <mergeCell ref="N37:P39"/>
     <mergeCell ref="X3:AC3"/>
-    <mergeCell ref="N5:P7"/>
+    <mergeCell ref="M33:M35"/>
+    <mergeCell ref="N21:P23"/>
     <mergeCell ref="H13:H15"/>
     <mergeCell ref="E3:G4"/>
+    <mergeCell ref="A25:C27"/>
     <mergeCell ref="AJ3:AO3"/>
-    <mergeCell ref="I13:I15"/>
+    <mergeCell ref="M17:M19"/>
+    <mergeCell ref="Q17:Q19"/>
     <mergeCell ref="E9:G11"/>
-    <mergeCell ref="R3:W3"/>
-    <mergeCell ref="A1:AO1"/>
     <mergeCell ref="M3:M4"/>
-    <mergeCell ref="I3:I4"/>
     <mergeCell ref="Q13:Q15"/>
     <mergeCell ref="N13:P15"/>
-    <mergeCell ref="H5:H7"/>
+    <mergeCell ref="A17:C19"/>
+    <mergeCell ref="M9:M11"/>
+    <mergeCell ref="Q37:Q39"/>
+    <mergeCell ref="Q21:Q23"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="H9:H11"/>
+    <mergeCell ref="E37:G39"/>
+    <mergeCell ref="N25:P27"/>
+    <mergeCell ref="M13:M15"/>
+    <mergeCell ref="E29:G31"/>
+    <mergeCell ref="E13:G15"/>
+    <mergeCell ref="H37:H39"/>
+    <mergeCell ref="Q25:Q27"/>
+    <mergeCell ref="N29:P31"/>
     <mergeCell ref="I9:I11"/>
-    <mergeCell ref="A5:C7"/>
-    <mergeCell ref="N3:P4"/>
-    <mergeCell ref="M9:M11"/>
-    <mergeCell ref="M5:M7"/>
-    <mergeCell ref="A13:C15"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="N9:P11"/>
-    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="A33:C35"/>
     <mergeCell ref="A3:C4"/>
-    <mergeCell ref="AD3:AI3"/>
     <mergeCell ref="Q5:Q7"/>
-    <mergeCell ref="AP3:AU3"/>
-    <mergeCell ref="H9:H11"/>
     <mergeCell ref="A2:AO2"/>
-    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="E33:G35"/>
     <mergeCell ref="A9:C11"/>
-    <mergeCell ref="Q3:Q4"/>
-    <mergeCell ref="M13:M15"/>
+    <mergeCell ref="Q29:Q31"/>
+    <mergeCell ref="I21:I23"/>
+    <mergeCell ref="M37:M39"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>

</xml_diff>